<commit_message>
📊 Horarios actualizados Línea 141 - 4208
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:18:55</t>
+          <t>Última actualización: 02:07:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -515,6 +515,81 @@
         <v>100</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:07:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>02:56</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>49</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>02:07:30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>03:48</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>101</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>02:07:30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>03:52</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>105</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -531,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,14 +619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:18:55</t>
+          <t>Última actualización: 02:07:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -602,6 +677,56 @@
         <v>54</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>02:07:30</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>02:56</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>49</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:07:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>03:52</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>105</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -631,7 +756,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:18:55</t>
+          <t>Última actualización: 02:07:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4209
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:07:30</t>
+          <t>Última actualización: 03:23:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>02:07:30</t>
+          <t>03:23:19</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>101</v>
+        <v>25</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>02:07:30</t>
+          <t>03:23:19</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -587,9 +587,134 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>105</v>
+        <v>29</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03:23:19</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>69</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>03:23:19</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>82</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>03:23:19</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>85</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>03:23:19</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>05:10</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>107</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>03:23:19</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>05:18</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>115</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -606,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,14 +744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:07:30</t>
+          <t>Última actualización: 03:23:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -710,7 +835,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:07:30</t>
+          <t>03:23:19</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -724,9 +849,34 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>105</v>
+        <v>29</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:23:19</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>85</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -756,7 +906,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:07:30</t>
+          <t>Última actualización: 03:23:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4210
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:23:19</t>
+          <t>Última actualización: 04:55:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>03:23:19</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>107</v>
+        <v>15</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>03:23:19</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -712,9 +712,434 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>115</v>
+        <v>23</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>05:25</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>30</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>05:35</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>40</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>05:43</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>48</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>49</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>05:53</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>58</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>06:03</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>68</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>80</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>06:17</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>82</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>06:20</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>85</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>06:23</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>88</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>06:24</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>89</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>06:32</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>97</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>06:33</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>86XR36_ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>98</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>06:38</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>103</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>06:46</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>111</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>06:49</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>84_ESC AGRARIA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>114</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>06:52</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>117</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -731,7 +1156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -744,14 +1169,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:23:19</t>
+          <t>Última actualización: 04:55:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -877,6 +1302,106 @@
         <v>85</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>05:35</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06:03</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>68</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:23</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>88</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:38</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>103</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -893,7 +1418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -906,14 +1431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:23:19</t>
+          <t>Última actualización: 04:55:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -966,6 +1491,81 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>05:34</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>39</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06:06</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>71</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:53</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>118</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4211
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:55:30</t>
+          <t>Última actualización: 05:55:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -848,12 +848,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>06:03</t>
+          <t>06:02</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>68</v>
+        <v>7</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -878,16 +878,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>06:15</t>
+          <t>06:03</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>06:17</t>
+          <t>06:14</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -928,16 +928,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>06:15</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,21 +948,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>06:23</t>
+          <t>06:17</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>06:24</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>89</v>
+        <v>25</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>06:32</t>
+          <t>06:22</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>97</v>
+        <v>27</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1028,16 +1028,16 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>06:33</t>
+          <t>06:23</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>06:38</t>
+          <t>06:24</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>103</v>
+        <v>29</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1078,16 +1078,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>06:46</t>
+          <t>06:32</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>06:49</t>
+          <t>06:32</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>84_ESC AGRARIA-ESC 49</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>114</v>
+        <v>37</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1128,18 +1128,618 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>06:33</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>86XR36_ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>98</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>06:38</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>43</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>50</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>06:46</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>111</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>06:48</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>84_ESC AGRARIA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>53</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>06:49</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>84_ESC AGRARIA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>114</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>06:52</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>117</v>
-      </c>
-      <c r="E32" t="inlineStr">
+      <c r="D38" t="n">
+        <v>57</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>06:56</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>61</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>06:57</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>62</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>07:03</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>17/64_OLMOS POR 520</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>68</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>07:04</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>69</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>07:08</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>73</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>77</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>07:13</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>78</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>07:17</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>82</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>07:18</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>83</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>85</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>07:23</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>88</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>89</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>07:29</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>94</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>96</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>101</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>07:42</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>107</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>07:46</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>111</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>113</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1156,7 +1756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1169,14 +1769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:55:30</t>
+          <t>Última actualización: 05:55:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -1335,12 +1935,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:03</t>
+          <t>06:02</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1349,7 +1949,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>68</v>
+        <v>7</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1365,7 +1965,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:23</t>
+          <t>06:03</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1374,7 +1974,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1385,23 +1985,98 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:22</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>27</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>04:55:30</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:23</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>88</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>06:38</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>103</v>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D15" t="n">
+        <v>43</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>77</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1418,7 +2093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1431,14 +2106,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:55:30</t>
+          <t>Última actualización: 05:55:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1522,12 +2197,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06:06</t>
+          <t>06:04</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1536,7 +2211,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>71</v>
+        <v>9</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1552,20 +2227,120 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>06:06</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>71</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06:52</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>57</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04:55:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>06:53</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>215D_LA PLATA</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D11" t="n">
         <v>118</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>07:09</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>74</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>92</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4212
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:55:52</t>
+          <t>Última actualización: 06:50:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 51</t>
+          <t>Total filas: 75</t>
         </is>
       </c>
     </row>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>06:52</t>
+          <t>06:50</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>84_ESC AGRARIA-ESC 49</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>06:56</t>
+          <t>06:52</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>61</v>
+        <v>2</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1328,16 +1328,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>06:57</t>
+          <t>06:56</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07:03</t>
+          <t>06:57</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>68</v>
+        <v>7</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07:04</t>
+          <t>06:57</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1403,16 +1403,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07:08</t>
+          <t>07:03</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>07:12</t>
+          <t>07:04</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1453,16 +1453,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>07:13</t>
+          <t>07:04</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>07:17</t>
+          <t>07:08</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>82</v>
+        <v>18</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>07:18</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1528,16 +1528,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:13</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>07:23</t>
+          <t>07:14</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>88</v>
+        <v>24</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>07:24</t>
+          <t>07:17</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:18</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>94</v>
+        <v>28</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1628,16 +1628,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>101</v>
+        <v>31</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1678,16 +1678,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07:42</t>
+          <t>07:23</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07:46</t>
+          <t>07:23</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>111</v>
+        <v>33</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1728,18 +1728,618 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>89</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>34</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>07:25</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>35</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>07:28</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>38</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>07:29</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>94</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>40</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>41</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>46</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>07:42</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>107</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>07:43</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>53</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>07:46</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>111</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>07:47</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>57</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>05:55:52</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>07:48</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D56" t="n">
+      <c r="D68" t="n">
         <v>113</v>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>59</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>07:56</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>66</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>08:03</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>73</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>08:04</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>74</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>08:07</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>77</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>89</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>91</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>08:23</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>93</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>103</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>104</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>08:43</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>113</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>118</v>
+      </c>
+      <c r="E80" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1756,7 +2356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1769,14 +2369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:55:52</t>
+          <t>Última actualización: 06:50:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2060,7 +2660,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2074,9 +2674,109 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07:28</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>38</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>103</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>104</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08:43</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>113</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2093,7 +2793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2106,14 +2806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:55:52</t>
+          <t>Última actualización: 06:50:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2247,12 +2947,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:52</t>
+          <t>06:50</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2261,7 +2961,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2272,12 +2972,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:53</t>
+          <t>06:52</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2286,7 +2986,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>118</v>
+        <v>57</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2297,50 +2997,150 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>07:09</t>
+          <t>06:53</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215D_LA PLATA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>74</v>
+        <v>118</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07:09</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>19</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>05:55:52</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>07:27</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D14" t="n">
         <v>92</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>58</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>08:24</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>94</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4213
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:50:36</t>
+          <t>Última actualización: 07:45:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 75</t>
+          <t>Total filas: 95</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1973,12 +1973,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>07:46</t>
+          <t>07:45</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>111</v>
+        <v>0</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,12 +1998,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>07:47</t>
+          <t>07:46</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>57</v>
+        <v>111</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>07:48</t>
+          <t>07:47</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>113</v>
+        <v>57</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,12 +2048,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>07:49</t>
+          <t>07:48</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2078,16 +2078,16 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>07:56</t>
+          <t>07:49</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>07:53</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>73</v>
+        <v>8</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>08:04</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>74</v>
+        <v>10</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2153,16 +2153,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>08:07</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:02</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>89</v>
+        <v>17</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>91</v>
+        <v>18</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>08:23</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>93</v>
+        <v>18</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2253,16 +2253,16 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>08:04</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>104</v>
+        <v>21</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2303,16 +2303,16 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>08:43</t>
+          <t>08:07</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,23 +2323,523 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>08:13</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>28</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>08:18</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>33</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
           <t>06:50:36</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>89</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>35</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>35</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>06:50:36</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>91</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>08:22</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>37</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>08:23</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>38</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>48</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>49</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>08:43</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>58</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
         <is>
           <t>08:48</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D80" t="n">
+      <c r="D91" t="n">
+        <v>63</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>66</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>77</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>78</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>09:13</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>88</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>91</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>93</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>96</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>105</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
         <v>118</v>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="E100" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2356,7 +2856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2369,14 +2869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:50:36</t>
+          <t>Última actualización: 07:45:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -2710,7 +3210,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2724,7 +3224,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>103</v>
+        <v>48</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2735,7 +3235,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2749,7 +3249,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>104</v>
+        <v>49</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2760,7 +3260,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2774,9 +3274,59 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>93</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>118</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2793,7 +3343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2806,14 +3356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:50:36</t>
+          <t>Última actualización: 07:45:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -3097,12 +3647,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:48</t>
+          <t>07:47</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3111,7 +3661,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3122,25 +3672,100 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>26</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>08:24</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>215C_ESC AGRARIA-LA PLATA</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>94</v>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="D19" t="n">
+        <v>39</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>71</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4214
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:E123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:45:53</t>
+          <t>Última actualización: 08:29:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 95</t>
+          <t>Total filas: 118</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>08:29</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2578,16 +2578,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>08:43</t>
+          <t>08:33</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2653,16 +2653,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>09:02</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>09:03</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>78</v>
+        <v>15</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>09:13</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>91</v>
+        <v>19</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2753,16 +2753,16 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>08:52</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2803,16 +2803,16 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>09:02</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>105</v>
+        <v>77</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2828,18 +2828,593 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>78</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>34</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>35</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>09:13</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>44</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>47</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>93</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>50</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>52</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>61</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>65</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>09:37</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>68</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
           <t>09:43</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C111" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D100" t="n">
+      <c r="D111" t="n">
         <v>118</v>
       </c>
-      <c r="E100" t="inlineStr">
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>75</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>76</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>89</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>95</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>10:06</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>97</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>10:06</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>97</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>103</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>10:14</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>105</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>111</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>112</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>115</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>116</v>
+      </c>
+      <c r="E123" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2856,7 +3431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2869,14 +3444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:45:53</t>
+          <t>Última actualización: 08:29:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3810,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3249,7 +3824,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3260,21 +3835,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>08:43</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>58</v>
+        <v>5</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3290,16 +3865,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3315,18 +3890,143 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>93</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>50</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>07:45:53</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>09:43</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D24" t="n">
         <v>118</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>75</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>95</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10:14</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>105</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3343,7 +4043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3356,14 +4056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:45:53</t>
+          <t>Última actualización: 08:29:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3747,7 +4447,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3761,9 +4461,109 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>43</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>96</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>109</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>112</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4215
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E123"/>
+  <dimension ref="A1:E140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:29:16</t>
+          <t>Última actualización: 09:07:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 118</t>
+          <t>Total filas: 135</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:13</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,12 +2973,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>50</v>
+        <v>93</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>52</v>
+        <v>11</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>65</v>
+        <v>14</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>09:37</t>
+          <t>09:28</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>118</v>
+        <v>23</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>75</v>
+        <v>27</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:36</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>76</v>
+        <v>29</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3178,16 +3178,16 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:37</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>10:06</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>10:06</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>97</v>
+        <v>38</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>10:12</t>
+          <t>09:48</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3303,16 +3303,16 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>10:14</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>111</v>
+        <v>57</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>10:21</t>
+          <t>10:06</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>112</v>
+        <v>59</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3378,16 +3378,16 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:06</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3403,18 +3403,443 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>103</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>10:14</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>67</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>111</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>74</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>77</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>77</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>08:29:16</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
           <t>10:25</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
+      <c r="C129" t="inlineStr">
         <is>
           <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
-      <c r="D123" t="n">
+      <c r="D129" t="n">
         <v>116</v>
       </c>
-      <c r="E123" t="inlineStr">
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>83</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>87</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>87</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>93</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>97</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>10:49</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>102</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>10:53</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>106</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>10:54</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>17/64_OLMOS POR 520</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>107</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>114</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>117</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>119</v>
+      </c>
+      <c r="E140" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3431,7 +3856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3444,14 +3869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:29:16</t>
+          <t>Última actualización: 09:07:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -3910,7 +4335,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3924,7 +4349,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3960,7 +4385,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3974,7 +4399,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -3985,7 +4410,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3999,7 +4424,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>95</v>
+        <v>57</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4010,7 +4435,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4024,9 +4449,34 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>105</v>
+        <v>67</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>87</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4043,7 +4493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4056,14 +4506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:29:16</t>
+          <t>Última actualización: 09:07:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4472,12 +4922,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>09:12</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4486,7 +4936,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -4502,70 +4952,120 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10:05</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10:18</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-40 Y 115</t>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>71</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>10:21</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>112</v>
-      </c>
-      <c r="E24" t="inlineStr">
+      <c r="D25" t="n">
+        <v>74</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>09:07:23</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>96</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4216
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E140"/>
+  <dimension ref="A1:E175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:07:23</t>
+          <t>Última actualización: 10:34:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 135</t>
+          <t>Total filas: 170</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>59</v>
+        <v>97</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>10:35</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>93</v>
+        <v>1</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:37</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3703,16 +3703,16 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>10:49</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>10:53</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>106</v>
+        <v>10</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>10:54</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>107</v>
+        <v>10</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>11:01</t>
+          <t>10:46</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>10:48</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>117</v>
+        <v>14</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,23 +3823,898 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>10:49</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>15</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
           <t>09:07:23</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr">
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>10:53</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>106</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>10:54</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>17/64_OLMOS POR 520</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>20</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>24</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>26</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>27</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>27</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>30</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
         <is>
           <t>11:06</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
+      <c r="C148" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D140" t="n">
+      <c r="D148" t="n">
+        <v>32</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>11:09</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>35</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>11:11</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>37</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>39</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>44</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>47</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>47</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>50</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>51</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>55</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>60</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>60</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>11:37</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>63</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>66</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>72</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>11:47</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>73</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>11:52</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>78</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>79</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>11:56</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>82</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>87</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>95</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>12:12</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>98</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>12:18</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>104</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>107</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>110</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>111</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
         <v>119</v>
       </c>
-      <c r="E140" t="inlineStr">
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>119</v>
+      </c>
+      <c r="E175" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3856,7 +4731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3869,14 +4744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:07:23</t>
+          <t>Última actualización: 10:34:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -4460,7 +5335,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4474,9 +5349,134 @@
         </is>
       </c>
       <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>47</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>50</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>60</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>72</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
         <v>87</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4493,7 +5493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4506,14 +5506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:07:23</t>
+          <t>Última actualización: 10:34:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -5047,7 +6047,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5061,9 +6061,84 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>96</v>
+        <v>9</v>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>44</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>12:06</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>92</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>10:34:33</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>95</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4217
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E175"/>
+  <dimension ref="A1:E194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:34:33</t>
+          <t>Última actualización: 11:33:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 170</t>
+          <t>Total filas: 189</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:33</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>11:37</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4353,16 +4353,16 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>11:37</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>11:46</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>11:47</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>73</v>
+        <v>7</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>78</v>
+        <v>7</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:46</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>79</v>
+        <v>13</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>11:56</t>
+          <t>11:47</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>11:47</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>12:09</t>
+          <t>11:50</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>12:12</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>98</v>
+        <v>19</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>12:18</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>104</v>
+        <v>19</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>107</v>
+        <v>20</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>11:54</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>111</v>
+        <v>22</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>11:56</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>119</v>
+        <v>23</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,23 +4698,498 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>25</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>27</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>28</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>12:06</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>33</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>36</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>12:12</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>39</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>41</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>12:18</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>45</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>48</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>51</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>52</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>59</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>60</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
           <t>10:34:33</t>
         </is>
       </c>
-      <c r="B175" t="inlineStr">
+      <c r="B188" t="inlineStr">
         <is>
           <t>12:33</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
+      <c r="C188" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D175" t="n">
+      <c r="D188" t="n">
         <v>119</v>
       </c>
-      <c r="E175" t="inlineStr">
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>67</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>68</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>12:48</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>75</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>12:49</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>76</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>100</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>108</v>
+      </c>
+      <c r="E194" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4744,7 +5219,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:34:33</t>
+          <t>Última actualización: 11:33:25</t>
         </is>
       </c>
     </row>
@@ -5410,7 +5885,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5424,7 +5899,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5435,7 +5910,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5449,7 +5924,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>72</v>
+        <v>13</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5460,7 +5935,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5474,7 +5949,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>87</v>
+        <v>28</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5493,7 +5968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5506,14 +5981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:34:33</t>
+          <t>Última actualización: 11:33:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6572,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -6111,7 +6586,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>92</v>
+        <v>33</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -6122,7 +6597,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6136,9 +6611,109 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>95</v>
+        <v>36</v>
       </c>
       <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>12:59</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>86</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>98</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>101</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>11:33:25</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>115</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4218
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E194"/>
+  <dimension ref="A1:E221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:33:25</t>
+          <t>Última actualización: 12:24:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 189</t>
+          <t>Total filas: 216</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,12 +4948,12 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5003,16 +5003,16 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:26</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>119</v>
+        <v>2</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>12:40</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>12:41</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>12:48</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>12:49</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>76</v>
+        <v>9</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,23 +5173,698 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>16</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>16</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
           <t>11:33:25</t>
         </is>
       </c>
-      <c r="B194" t="inlineStr">
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>68</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>21</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>12:48</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>24</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>12:49</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>25</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>26</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>12:59</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>35</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>36</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>46</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>49</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>53</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>55</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
         <is>
           <t>13:21</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr">
+      <c r="C207" t="inlineStr">
         <is>
           <t>26_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D194" t="n">
-        <v>108</v>
-      </c>
-      <c r="E194" t="inlineStr">
+      <c r="D207" t="n">
+        <v>57</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>61</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>77</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>13:48</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>84</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>89</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>90</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>93</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>96</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>101</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>102</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>109</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>113</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>114</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>115</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>117</v>
+      </c>
+      <c r="E221" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5206,7 +5881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5219,14 +5894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:33:25</t>
+          <t>Última actualización: 12:24:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -5952,6 +6627,81 @@
         <v>28</v>
       </c>
       <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>12:26</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>61</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>102</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5968,7 +6718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5981,14 +6731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:33:25</t>
+          <t>Última actualización: 12:24:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -6622,7 +7372,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6636,7 +7386,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -6647,7 +7397,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6661,7 +7411,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>98</v>
+        <v>47</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -6672,7 +7422,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6686,7 +7436,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6697,7 +7447,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6711,11 +7461,36 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>115</v>
+        <v>64</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>80</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4219
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E221"/>
+  <dimension ref="A1:E242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:24:23</t>
+          <t>Última actualización: 13:10:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 216</t>
+          <t>Total filas: 237</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>59</v>
+        <v>97</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>9</v>
+        <v>119</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>13:12</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>13:12</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>53</v>
+        <v>2</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,12 +5473,12 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>13:19</t>
+          <t>13:12</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>55</v>
+        <v>2</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5503,16 +5503,16 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:16</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>61</v>
+        <v>6</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,12 +5548,12 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>13:41</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -5562,7 +5562,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>77</v>
+        <v>7</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5578,16 +5578,16 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>13:48</t>
+          <t>13:19</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>13:53</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>89</v>
+        <v>11</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>90</v>
+        <v>11</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>13:57</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>96</v>
+        <v>14</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>14:06</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>102</v>
+        <v>15</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5753,16 +5753,16 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>109</v>
+        <v>61</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:29</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>113</v>
+        <v>19</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>14:18</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>114</v>
+        <v>21</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>13:36</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>115</v>
+        <v>26</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,23 +5848,548 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>31</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>13:42</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>32</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
           <t>12:24:23</t>
         </is>
       </c>
-      <c r="B221" t="inlineStr">
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>13:48</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>84</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>43</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>44</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>47</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>50</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>55</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>56</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>14:12</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>62</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>12:24:23</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>109</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>67</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>68</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>69</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
         <is>
           <t>14:21</t>
         </is>
       </c>
-      <c r="C221" t="inlineStr">
+      <c r="C235" t="inlineStr">
         <is>
           <t>26_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D221" t="n">
-        <v>117</v>
-      </c>
-      <c r="E221" t="inlineStr">
+      <c r="D235" t="n">
+        <v>71</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>77</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>80</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>85</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>92</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>104</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>110</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>111</v>
+      </c>
+      <c r="E242" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5881,7 +6406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5894,14 +6419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:24:23</t>
+          <t>Última actualización: 13:10:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -6660,12 +7185,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -6674,7 +7199,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>61</v>
+        <v>14</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6690,18 +7215,93 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>61</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>14:06</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>102</v>
-      </c>
-      <c r="E36" t="inlineStr">
+      <c r="D37" t="n">
+        <v>56</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>80</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>110</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6718,7 +7318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6731,14 +7331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:24:23</t>
+          <t>Última actualización: 13:10:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -7422,21 +8022,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:12</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -7447,25 +8047,25 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>64</v>
+        <v>4</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
@@ -7477,18 +8077,68 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>64</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>19</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>13:10:41</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>13:44</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>80</v>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D36" t="n">
+        <v>34</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4220
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E242"/>
+  <dimension ref="A1:E265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:41</t>
+          <t>Última actualización: 14:11:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 237</t>
+          <t>Total filas: 260</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>9</v>
+        <v>119</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,12 +6098,12 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -6112,7 +6112,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>109</v>
+        <v>62</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>67</v>
+        <v>2</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>14:18</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>14:18</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>14:21</t>
+          <t>14:18</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>71</v>
+        <v>7</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:19</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>77</v>
+        <v>8</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:21</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>14:42</t>
+          <t>14:29</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>92</v>
+        <v>18</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>104</v>
+        <v>19</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>110</v>
+        <v>22</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,23 +6373,598 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>24</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>30</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>31</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>43</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>44</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
           <t>13:10:41</t>
         </is>
       </c>
-      <c r="B242" t="inlineStr">
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>110</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
         <is>
           <t>15:01</t>
         </is>
       </c>
-      <c r="C242" t="inlineStr">
+      <c r="C248" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D242" t="n">
-        <v>111</v>
-      </c>
-      <c r="E242" t="inlineStr">
+      <c r="D248" t="n">
+        <v>50</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>50</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>58</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>15:17</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>66</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>67</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>15:21</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>70</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>71</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>71</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>79</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>15:33</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>82</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>89</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>94</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>98</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>107</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>109</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>109</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>114</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>16:06</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>115</v>
+      </c>
+      <c r="E265" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6406,7 +6981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6419,14 +6994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:41</t>
+          <t>Última actualización: 14:11:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -7260,7 +7835,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7274,7 +7849,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>80</v>
+        <v>19</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -7302,6 +7877,106 @@
         <v>110</v>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>50</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>58</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>89</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>94</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7318,7 +7993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7331,14 +8006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:41</t>
+          <t>Última actualización: 14:11:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -8141,6 +8816,106 @@
       <c r="E36" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>59</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>15:36</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>85</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>14:11:32</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>109</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4221
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E265"/>
+  <dimension ref="A1:E289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:11:32</t>
+          <t>Última actualización: 15:06:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 260</t>
+          <t>Total filas: 284</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>9</v>
+        <v>119</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>15:09</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>15:17</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>15:21</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6678,16 +6678,16 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:09</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:17</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>71</v>
+        <v>11</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6728,16 +6728,16 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>15:33</t>
+          <t>15:21</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>82</v>
+        <v>15</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>15:21</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>89</v>
+        <v>15</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,21 +6798,21 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>94</v>
+        <v>16</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6828,16 +6828,16 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>15:49</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>98</v>
+        <v>71</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>107</v>
+        <v>20</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,21 +6873,21 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:33</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>109</v>
+        <v>27</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>114</v>
+        <v>34</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,23 +6948,623 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
+          <t>15:42</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>36</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>39</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>43</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>52</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>54</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>54</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>59</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
           <t>16:06</t>
         </is>
       </c>
-      <c r="C265" t="inlineStr">
+      <c r="C272" t="inlineStr">
         <is>
           <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
-      <c r="D265" t="n">
-        <v>115</v>
-      </c>
-      <c r="E265" t="inlineStr">
+      <c r="D272" t="n">
+        <v>60</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>64</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>68</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>16:20</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>74</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>16:21</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>75</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>16:21</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>75</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>16:27</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>81</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>16:28</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>11_ESC 3-ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>82</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>16:39</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>93</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>94</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>98</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>99</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>100</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>16:49</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>103</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>109</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>109</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>16:58</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>112</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>119</v>
+      </c>
+      <c r="E289" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6981,7 +7581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6994,14 +7594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:11:32</t>
+          <t>Última actualización: 15:06:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -7910,12 +8510,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>15:09</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -7924,7 +8524,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7940,16 +8540,16 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>15:09</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>89</v>
+        <v>58</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7960,23 +8560,98 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>34</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>15:45</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>94</v>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D44" t="n">
+        <v>39</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>98</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>109</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7993,7 +8668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8006,14 +8681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:11:32</t>
+          <t>Última actualización: 15:06:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -8872,50 +9547,125 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>15:36</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>15:36</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>30</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215D_LA PLATA</t>
         </is>
       </c>
-      <c r="D40" t="n">
-        <v>109</v>
-      </c>
-      <c r="E40" t="inlineStr">
+      <c r="D41" t="n">
+        <v>54</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>98</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>15:06:33</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>16:52</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>106</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4222
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E289"/>
+  <dimension ref="A1:E312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:06:33</t>
+          <t>Última actualización: 16:07:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 284</t>
+          <t>Total filas: 307</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>9</v>
+        <v>119</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6758,7 +6758,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
@@ -6783,7 +6783,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,21 +7173,21 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>16:20</t>
+          <t>16:13</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>74</v>
+        <v>6</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>75</v>
+        <v>7</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:17</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>16:27</t>
+          <t>16:20</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7303,16 +7303,16 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>16:28</t>
+          <t>16:20</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>11_ESC 3-ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,21 +7323,21 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>16:39</t>
+          <t>16:21</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>93</v>
+        <v>14</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:21</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>94</v>
+        <v>14</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>98</v>
+        <v>16</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7403,16 +7403,16 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>16:27</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:28</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ESC 3-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>100</v>
+        <v>21</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>16:49</t>
+          <t>16:37</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>103</v>
+        <v>30</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:39</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>109</v>
+        <v>32</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>109</v>
+        <v>33</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>16:58</t>
+          <t>16:42</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>112</v>
+        <v>35</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,23 +7548,598 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>37</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>38</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>38</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
           <t>15:06:33</t>
         </is>
       </c>
-      <c r="B289" t="inlineStr">
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>100</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>16:49</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>42</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>48</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>48</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>16:58</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>51</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>52</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>57</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
         <is>
           <t>17:05</t>
         </is>
       </c>
-      <c r="C289" t="inlineStr">
+      <c r="C299" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D289" t="n">
-        <v>119</v>
-      </c>
-      <c r="E289" t="inlineStr">
+      <c r="D299" t="n">
+        <v>58</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>17:09</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>62</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>63</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>63</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>17:20</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>73</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>74</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>84</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>17:34</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>87</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>93</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>100</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>105</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>17:56</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>109</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>113</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>118</v>
+      </c>
+      <c r="E312" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7581,7 +8156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7594,14 +8169,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:06:33</t>
+          <t>Última actualización: 16:07:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -8610,7 +9185,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8624,7 +9199,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>98</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -8635,7 +9210,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8649,9 +9224,34 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>109</v>
+        <v>48</v>
       </c>
       <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>63</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8668,7 +9268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8681,14 +9281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:06:33</t>
+          <t>Última actualización: 16:07:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -9622,7 +10222,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -9636,7 +10236,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>98</v>
+        <v>37</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -9647,7 +10247,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -9661,9 +10261,59 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>106</v>
+        <v>45</v>
       </c>
       <c r="E43" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>67</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>17:27</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>80</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4223
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E312"/>
+  <dimension ref="A1:E339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:07:47</t>
+          <t>Última actualización: 16:52:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 307</t>
+          <t>Total filas: 334</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>9</v>
+        <v>119</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7708,7 +7708,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:58</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,21 +7773,21 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>16:58</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7803,16 +7803,16 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,12 +7823,12 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>17:09</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -7837,7 +7837,7 @@
         </is>
       </c>
       <c r="D300" t="n">
-        <v>62</v>
+        <v>8</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,21 +7848,21 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>63</v>
+        <v>11</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7873,21 +7873,21 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>63</v>
+        <v>12</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,21 +7898,21 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7928,16 +7928,16 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:09</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7953,16 +7953,16 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7978,16 +7978,16 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>17:34</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,21 +7998,21 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>93</v>
+        <v>18</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>105</v>
+        <v>19</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,21 +8073,21 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>17:56</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>109</v>
+        <v>19</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8103,16 +8103,16 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>113</v>
+        <v>73</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,23 +8123,698 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>29</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>29</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>31</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>17:27</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>35</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
           <t>16:07:47</t>
         </is>
       </c>
-      <c r="B312" t="inlineStr">
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>84</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>40</v>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>17:34</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>87</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>43</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>48</v>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>55</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>105</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>17:56</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>109</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>17:57</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>65</v>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>17:57</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>65</v>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>113</v>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>18:01</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>69</v>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>16:07:47</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
         <is>
           <t>18:05</t>
         </is>
       </c>
-      <c r="C312" t="inlineStr">
+      <c r="C328" t="inlineStr">
         <is>
           <t>83_ALUAR</t>
         </is>
       </c>
-      <c r="D312" t="n">
+      <c r="D328" t="n">
         <v>118</v>
       </c>
-      <c r="E312" t="inlineStr">
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>18:06</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D329" t="n">
+        <v>74</v>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>18:09</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D330" t="n">
+        <v>77</v>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>89</v>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D332" t="n">
+        <v>93</v>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D333" t="n">
+        <v>98</v>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>99</v>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D335" t="n">
+        <v>100</v>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>108</v>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D337" t="n">
+        <v>110</v>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>18:47</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>115</v>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>18:49</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D339" t="n">
+        <v>117</v>
+      </c>
+      <c r="E339" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8156,7 +8831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8169,14 +8844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:07:47</t>
+          <t>Última actualización: 16:52:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -9210,7 +9885,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -9224,7 +9899,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -9252,6 +9927,106 @@
         <v>63</v>
       </c>
       <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>17:11</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>19</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>110</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>18:47</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>115</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>18:49</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>117</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9268,7 +10043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9281,14 +10056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:07:47</t>
+          <t>Última actualización: 16:52:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -10247,7 +11022,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10261,7 +11036,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -10297,23 +11072,123 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>23</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>16:07:47</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>17:27</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D45" t="n">
+      <c r="D46" t="n">
         <v>80</v>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>17:28</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>36</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>110</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>118</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4224
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E339"/>
+  <dimension ref="A1:E358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:52:07</t>
+          <t>Última actualización: 17:19:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 334</t>
+          <t>Total filas: 353</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>9</v>
+        <v>119</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D297" t="n">
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7983,11 +7983,11 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8023,7 +8023,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -8033,11 +8033,11 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8098,12 +8098,12 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>17:19</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -8112,7 +8112,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,12 +8123,12 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -8137,7 +8137,7 @@
         </is>
       </c>
       <c r="D312" t="n">
-        <v>29</v>
+        <v>73</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8178,16 +8178,16 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,21 +8198,21 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>17:27</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8248,21 +8248,21 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8273,21 +8273,21 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>17:34</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>87</v>
+        <v>7</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8303,16 +8303,16 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:27</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8323,21 +8323,21 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8353,16 +8353,16 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8373,21 +8373,21 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -8403,16 +8403,16 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>17:56</t>
+          <t>17:34</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>109</v>
+        <v>87</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,21 +8423,21 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>17:57</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>65</v>
+        <v>16</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8448,21 +8448,21 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>17:57</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>65</v>
+        <v>19</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,21 +8473,21 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8498,21 +8498,21 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>18:01</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>69</v>
+        <v>28</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8528,16 +8528,16 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,21 +8548,21 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>18:06</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8573,21 +8573,21 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>18:09</t>
+          <t>17:56</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>77</v>
+        <v>37</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8603,16 +8603,16 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>17:57</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8628,16 +8628,16 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>17:57</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>93</v>
+        <v>65</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8648,21 +8648,21 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,12 +8673,12 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -8687,7 +8687,7 @@
         </is>
       </c>
       <c r="D334" t="n">
-        <v>99</v>
+        <v>42</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,21 +8698,21 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>18:32</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,21 +8723,21 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>108</v>
+        <v>47</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,21 +8748,21 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>18:42</t>
+          <t>18:09</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>110</v>
+        <v>50</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8773,21 +8773,21 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>18:47</t>
+          <t>18:16</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>115</v>
+        <v>57</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,23 +8798,498 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>18:16</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D339" t="n">
+        <v>57</v>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>62</v>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>65</v>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
           <t>16:52:07</t>
         </is>
       </c>
-      <c r="B339" t="inlineStr">
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>93</v>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>71</v>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>72</v>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>72</v>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D346" t="n">
+        <v>100</v>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D347" t="n">
+        <v>81</v>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>83</v>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>18:46</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>87</v>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>18:47</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
+        <v>115</v>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>89</v>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
         <is>
           <t>18:49</t>
         </is>
       </c>
-      <c r="C339" t="inlineStr">
+      <c r="C352" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D339" t="n">
+      <c r="D352" t="n">
         <v>117</v>
       </c>
-      <c r="E339" t="inlineStr">
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>96</v>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>106</v>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>19:06</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>107</v>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>109</v>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>116</v>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>119</v>
+      </c>
+      <c r="E358" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8831,7 +9306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8844,14 +9319,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:52:07</t>
+          <t>Última actualización: 17:19:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 49</t>
         </is>
       </c>
     </row>
@@ -9220,7 +9695,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -9245,7 +9720,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -9960,7 +10435,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -9974,7 +10449,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>110</v>
+        <v>83</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -9985,12 +10460,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>18:47</t>
+          <t>18:46</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -9999,7 +10474,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -10015,18 +10490,93 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>18:47</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>115</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>89</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>18:49</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D53" t="n">
         <v>117</v>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>119</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10043,7 +10593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10056,14 +10606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:52:07</t>
+          <t>Última actualización: 17:19:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -11097,7 +11647,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -11111,7 +11661,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -11147,7 +11697,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -11161,7 +11711,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>110</v>
+        <v>83</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -11172,23 +11722,73 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>18:49</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>90</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>16:52:07</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D49" t="n">
+      <c r="D50" t="n">
         <v>118</v>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>17:19:27</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>95</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4225
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E358"/>
+  <dimension ref="A1:E373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:19:27</t>
+          <t>Última actualización: 17:48:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 353</t>
+          <t>Total filas: 368</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6758,7 +6758,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
@@ -6783,7 +6783,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -7273,7 +7273,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -7283,11 +7283,11 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7308,11 +7308,11 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D297" t="n">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -7998,7 +7998,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -8008,11 +8008,11 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8173,7 +8173,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -8183,11 +8183,11 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,7 +8198,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -8208,11 +8208,11 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8523,21 +8523,21 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:49</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>105</v>
+        <v>1</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,21 +8548,21 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:49</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8573,21 +8573,21 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>17:56</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8598,12 +8598,12 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>17:57</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -8612,7 +8612,7 @@
         </is>
       </c>
       <c r="D331" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8623,21 +8623,21 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>17:57</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8648,21 +8648,21 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:56</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>113</v>
+        <v>37</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,21 +8673,21 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>18:01</t>
+          <t>17:56</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,21 +8698,21 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:57</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>118</v>
+        <v>65</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,21 +8723,21 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>18:06</t>
+          <t>17:57</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,21 +8748,21 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>18:09</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8778,16 +8778,16 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>18:16</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,21 +8798,21 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>18:16</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>57</v>
+        <v>13</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8823,21 +8823,21 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,21 +8873,21 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:09</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>93</v>
+        <v>50</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,21 +8898,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:09</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>18:16</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8953,16 +8953,16 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>18:16</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,21 +8973,21 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>18:32</t>
+          <t>18:18</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -9003,16 +9003,16 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9023,21 +9023,21 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>18:42</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>83</v>
+        <v>35</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9048,21 +9048,21 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>18:46</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9078,16 +9078,16 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>18:47</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>115</v>
+        <v>93</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9103,16 +9103,16 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>18:48</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9123,21 +9123,21 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>18:49</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>117</v>
+        <v>72</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9148,21 +9148,21 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9173,21 +9173,21 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:32</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9198,21 +9198,21 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>19:06</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>107</v>
+        <v>49</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9223,21 +9223,21 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:40</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>109</v>
+        <v>52</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -9248,21 +9248,21 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>18:42</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>116</v>
+        <v>54</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -9273,23 +9273,398 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
+          <t>18:46</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>58</v>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>18:47</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>115</v>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D360" t="n">
+        <v>60</v>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>18:49</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>117</v>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>67</v>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>77</v>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>19:06</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>78</v>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>80</v>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>87</v>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
           <t>19:18</t>
         </is>
       </c>
-      <c r="C358" t="inlineStr">
+      <c r="C367" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D358" t="n">
-        <v>119</v>
-      </c>
-      <c r="E358" t="inlineStr">
+      <c r="D367" t="n">
+        <v>90</v>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>90</v>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>93</v>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>100</v>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>102</v>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>19:39</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D372" t="n">
+        <v>111</v>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>118</v>
+      </c>
+      <c r="E373" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9319,7 +9694,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:19:27</t>
+          <t>Última actualización: 17:48:37</t>
         </is>
       </c>
     </row>
@@ -9695,7 +10070,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -9720,7 +10095,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -10435,7 +10810,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -10449,7 +10824,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>83</v>
+        <v>54</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -10460,7 +10835,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -10474,7 +10849,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -10510,7 +10885,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -10524,7 +10899,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>89</v>
+        <v>60</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -10560,7 +10935,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10574,7 +10949,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>119</v>
+        <v>90</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -10593,7 +10968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10606,14 +10981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:19:27</t>
+          <t>Última actualización: 17:48:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -11697,12 +12072,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>18:42</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -11711,7 +12086,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>83</v>
+        <v>53</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -11727,32 +12102,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>18:49</t>
+          <t>18:42</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:49</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -11761,7 +12136,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>118</v>
+        <v>61</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -11772,23 +12147,48 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>118</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>17:48:37</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>18:54</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D51" t="n">
-        <v>95</v>
-      </c>
-      <c r="E51" t="inlineStr">
+      <c r="D52" t="n">
+        <v>66</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4226
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E373"/>
+  <dimension ref="A1:E383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:48:37</t>
+          <t>Última actualización: 18:06:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 368</t>
+          <t>Total filas: 378</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>59</v>
+        <v>97</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6798,7 +6798,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -6808,11 +6808,11 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -6833,11 +6833,11 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D297" t="n">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8023,7 +8023,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -8033,11 +8033,11 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8173,7 +8173,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -8183,11 +8183,11 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,7 +8198,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -8208,11 +8208,11 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8648,7 +8648,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -8658,11 +8658,11 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,7 +8673,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -8683,11 +8683,11 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D336" t="n">
@@ -8848,7 +8848,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -8862,7 +8862,7 @@
         </is>
       </c>
       <c r="D341" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,21 +8873,21 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>18:09</t>
+          <t>18:07</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,21 +8898,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>18:09</t>
+          <t>18:07</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>18:16</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,12 +8948,12 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>18:16</t>
+          <t>18:09</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -8962,7 +8962,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,21 +8973,21 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>18:18</t>
+          <t>18:09</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,21 +8998,21 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:09</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>62</v>
+        <v>3</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9023,21 +9023,21 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9048,21 +9048,21 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,21 +9073,21 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:16</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,21 +9098,21 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:16</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9123,21 +9123,21 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>18:17</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9153,16 +9153,16 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>18:18</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9173,21 +9173,21 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>18:32</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9198,12 +9198,12 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -9212,7 +9212,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9223,21 +9223,21 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -9248,21 +9248,21 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>18:42</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>54</v>
+        <v>93</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -9273,21 +9273,21 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>18:46</t>
+          <t>18:27</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -9298,21 +9298,21 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>18:47</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>115</v>
+        <v>71</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -9323,21 +9323,21 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>18:48</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9348,21 +9348,21 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>18:49</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>117</v>
+        <v>25</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -9373,21 +9373,21 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:32</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>67</v>
+        <v>100</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9403,16 +9403,16 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -9423,21 +9423,21 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>19:06</t>
+          <t>18:40</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -9448,21 +9448,21 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:42</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>80</v>
+        <v>36</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -9473,21 +9473,21 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>18:46</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>87</v>
+        <v>40</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -9498,21 +9498,21 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>18:47</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -9523,21 +9523,21 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>18:48</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -9548,21 +9548,21 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>18:49</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -9573,21 +9573,21 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -9598,21 +9598,21 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -9623,21 +9623,21 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>19:39</t>
+          <t>19:06</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>111</v>
+        <v>60</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -9653,18 +9653,268 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>80</v>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>19:09</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D374" t="n">
+        <v>63</v>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>69</v>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>72</v>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>72</v>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>75</v>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>82</v>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D380" t="n">
+        <v>84</v>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>19:39</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D381" t="n">
+        <v>93</v>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
           <t>19:46</t>
         </is>
       </c>
-      <c r="C373" t="inlineStr">
+      <c r="C382" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D373" t="n">
-        <v>118</v>
-      </c>
-      <c r="E373" t="inlineStr">
+      <c r="D382" t="n">
+        <v>100</v>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>116</v>
+      </c>
+      <c r="E383" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9694,7 +9944,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:48:37</t>
+          <t>Última actualización: 18:06:31</t>
         </is>
       </c>
     </row>
@@ -10070,7 +10320,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -10095,7 +10345,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -10810,7 +11060,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -10824,7 +11074,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -10835,7 +11085,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -10849,7 +11099,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -10885,7 +11135,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -10899,7 +11149,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -10935,7 +11185,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10949,7 +11199,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -10981,7 +11231,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:48:37</t>
+          <t>Última actualización: 18:06:31</t>
         </is>
       </c>
     </row>
@@ -12097,7 +12347,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -12111,7 +12361,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -12122,7 +12372,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -12136,7 +12386,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -12172,7 +12422,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -12186,7 +12436,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4227
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E383"/>
+  <dimension ref="A1:E405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:06:31</t>
+          <t>Última actualización: 18:34:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 378</t>
+          <t>Total filas: 400</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>59</v>
+        <v>97</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>9</v>
+        <v>119</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -6758,7 +6758,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
@@ -6783,7 +6783,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -6798,7 +6798,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -6808,11 +6808,11 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -6833,11 +6833,11 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7273,7 +7273,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -7283,11 +7283,11 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7308,11 +7308,11 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -7998,7 +7998,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -8008,11 +8008,11 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,7 +8023,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -8033,11 +8033,11 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8123,7 +8123,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -8133,11 +8133,11 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,7 +8148,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -8158,11 +8158,11 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D336" t="n">
@@ -9398,21 +9398,21 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -9423,21 +9423,21 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -9448,21 +9448,21 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>18:42</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -9473,21 +9473,21 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>18:46</t>
+          <t>18:40</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -9498,21 +9498,21 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>18:47</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>115</v>
+        <v>7</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -9528,16 +9528,16 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>18:48</t>
+          <t>18:42</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -9548,21 +9548,21 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>18:49</t>
+          <t>18:45</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>117</v>
+        <v>11</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -9573,21 +9573,21 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:46</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -9598,21 +9598,21 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:47</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -9623,21 +9623,21 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>19:06</t>
+          <t>18:48</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -9648,21 +9648,21 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:49</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>80</v>
+        <v>117</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -9673,21 +9673,21 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>19:09</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>63</v>
+        <v>17</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -9698,21 +9698,21 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -9723,21 +9723,21 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -9748,21 +9748,21 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -9778,16 +9778,16 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="E378" t="inlineStr">
         <is>
@@ -9803,16 +9803,16 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>19:06</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="E379" t="inlineStr">
         <is>
@@ -9823,21 +9823,21 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D380" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E380" t="inlineStr">
         <is>
@@ -9848,21 +9848,21 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>19:39</t>
+          <t>19:09</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>93</v>
+        <v>35</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9873,21 +9873,21 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E382" t="inlineStr">
         <is>
@@ -9903,18 +9903,568 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>69</v>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D384" t="n">
+        <v>43</v>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D385" t="n">
+        <v>72</v>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D386" t="n">
+        <v>72</v>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>19:20</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D387" t="n">
+        <v>46</v>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D388" t="n">
+        <v>75</v>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D389" t="n">
+        <v>48</v>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>19:27</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D390" t="n">
+        <v>53</v>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D391" t="n">
+        <v>82</v>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>19:29</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D392" t="n">
+        <v>55</v>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D393" t="n">
+        <v>84</v>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>19:39</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>65</v>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D395" t="n">
+        <v>71</v>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D396" t="n">
+        <v>71</v>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D397" t="n">
+        <v>100</v>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D398" t="n">
+        <v>87</v>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>18:06:31</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
           <t>20:02</t>
         </is>
       </c>
-      <c r="C383" t="inlineStr">
+      <c r="C399" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D383" t="n">
+      <c r="D399" t="n">
         <v>116</v>
       </c>
-      <c r="E383" t="inlineStr">
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D400" t="n">
+        <v>91</v>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D401" t="n">
+        <v>92</v>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>20:17</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>103</v>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D403" t="n">
+        <v>109</v>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D404" t="n">
+        <v>109</v>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>20:28</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>114</v>
+      </c>
+      <c r="E405" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9931,7 +10481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9944,14 +10494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:06:31</t>
+          <t>Última actualización: 18:34:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 49</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -11060,12 +11610,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>18:42</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -11074,7 +11624,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -11090,16 +11640,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>18:46</t>
+          <t>18:42</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -11110,12 +11660,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>18:47</t>
+          <t>18:46</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -11124,7 +11674,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>115</v>
+        <v>12</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -11135,21 +11685,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>18:48</t>
+          <t>18:47</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>42</v>
+        <v>115</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -11160,12 +11710,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>18:49</t>
+          <t>18:48</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -11174,7 +11724,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>117</v>
+        <v>14</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -11185,23 +11735,73 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>16:52:07</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>18:49</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>117</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>43</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>18:06:31</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>19:18</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D54" t="n">
+      <c r="D56" t="n">
         <v>72</v>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11218,7 +11818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11231,14 +11831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:06:31</t>
+          <t>Última actualización: 18:34:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -12322,7 +12922,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -12336,7 +12936,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -12372,7 +12972,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -12386,7 +12986,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -12439,6 +13039,81 @@
         <v>48</v>
       </c>
       <c r="E52" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>18:56</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>22</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>20:17</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>103</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>20:28</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>114</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4228
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E405"/>
+  <dimension ref="A1:E421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:34:49</t>
+          <t>Última actualización: 18:53:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 400</t>
+          <t>Total filas: 416</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>9</v>
+        <v>119</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7273,7 +7273,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -7283,11 +7283,11 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7308,11 +7308,11 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D297" t="n">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7998,7 +7998,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -8008,11 +8008,11 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8033,7 +8033,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D308" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8173,7 +8173,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -8183,11 +8183,11 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,7 +8198,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -8208,11 +8208,11 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D336" t="n">
@@ -8773,7 +8773,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -8783,11 +8783,11 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,7 +8798,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -8808,11 +8808,11 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8883,7 +8883,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D342" t="n">
@@ -8908,7 +8908,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D343" t="n">
@@ -8973,7 +8973,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -8983,11 +8983,11 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -9008,11 +9008,11 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9333,7 +9333,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D360" t="n">
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9698,21 +9698,21 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -9723,21 +9723,21 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -9748,21 +9748,21 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -9773,21 +9773,21 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>59</v>
+        <v>2</v>
       </c>
       <c r="E378" t="inlineStr">
         <is>
@@ -9798,21 +9798,21 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>19:06</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="E379" t="inlineStr">
         <is>
@@ -9823,21 +9823,21 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D380" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="E380" t="inlineStr">
         <is>
@@ -9848,21 +9848,21 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>19:09</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9878,16 +9878,16 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="E382" t="inlineStr">
         <is>
@@ -9898,21 +9898,21 @@
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>19:06</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="E383" t="inlineStr">
         <is>
@@ -9923,21 +9923,21 @@
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="E384" t="inlineStr">
         <is>
@@ -9948,21 +9948,21 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:09</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="E385" t="inlineStr">
         <is>
@@ -9973,21 +9973,21 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D386" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E386" t="inlineStr">
         <is>
@@ -10003,16 +10003,16 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="E387" t="inlineStr">
         <is>
@@ -10023,21 +10023,21 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>75</v>
+        <v>22</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10053,16 +10053,16 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10073,21 +10073,21 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D390" t="n">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="E390" t="inlineStr">
         <is>
@@ -10098,21 +10098,21 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D391" t="n">
-        <v>82</v>
+        <v>25</v>
       </c>
       <c r="E391" t="inlineStr">
         <is>
@@ -10128,16 +10128,16 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>19:29</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,21 +10148,21 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10178,16 +10178,16 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>19:39</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D394" t="n">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="E394" t="inlineStr">
         <is>
@@ -10203,16 +10203,16 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D395" t="n">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="E395" t="inlineStr">
         <is>
@@ -10223,21 +10223,21 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>19:28</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D396" t="n">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="E396" t="inlineStr">
         <is>
@@ -10248,21 +10248,21 @@
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D397" t="n">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="E397" t="inlineStr">
         <is>
@@ -10273,12 +10273,12 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
@@ -10287,7 +10287,7 @@
         </is>
       </c>
       <c r="D398" t="n">
-        <v>87</v>
+        <v>37</v>
       </c>
       <c r="E398" t="inlineStr">
         <is>
@@ -10298,21 +10298,21 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:39</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>116</v>
+        <v>46</v>
       </c>
       <c r="E399" t="inlineStr">
         <is>
@@ -10323,12 +10323,12 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>19:42</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -10337,7 +10337,7 @@
         </is>
       </c>
       <c r="D400" t="n">
-        <v>91</v>
+        <v>49</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -10353,16 +10353,16 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D401" t="n">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="E401" t="inlineStr">
         <is>
@@ -10378,16 +10378,16 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D402" t="n">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="E402" t="inlineStr">
         <is>
@@ -10398,21 +10398,21 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="E403" t="inlineStr">
         <is>
@@ -10423,21 +10423,21 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D404" t="n">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="E404" t="inlineStr">
         <is>
@@ -10453,18 +10453,418 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>87</v>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D406" t="n">
+        <v>69</v>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D407" t="n">
+        <v>91</v>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D408" t="n">
+        <v>73</v>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D409" t="n">
+        <v>73</v>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>73</v>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>82</v>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>20:17</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D412" t="n">
+        <v>103</v>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>85</v>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>85</v>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>20:21</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>88</v>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D416" t="n">
+        <v>109</v>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D417" t="n">
+        <v>109</v>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
           <t>20:28</t>
         </is>
       </c>
-      <c r="C405" t="inlineStr">
+      <c r="C418" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D405" t="n">
-        <v>114</v>
-      </c>
-      <c r="E405" t="inlineStr">
+      <c r="D418" t="n">
+        <v>95</v>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>20:33</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D419" t="n">
+        <v>100</v>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D420" t="n">
+        <v>109</v>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>20:48</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>115</v>
+      </c>
+      <c r="E421" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10481,7 +10881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10494,14 +10894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:34:49</t>
+          <t>Última actualización: 18:53:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 51</t>
+          <t>Total filas: 55</t>
         </is>
       </c>
     </row>
@@ -11760,21 +12160,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -11785,23 +12185,123 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>43</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>19:18</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D56" t="n">
-        <v>72</v>
-      </c>
-      <c r="E56" t="inlineStr">
+      <c r="D57" t="n">
+        <v>25</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>20:33</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>100</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>109</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>20:48</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>115</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11818,7 +12318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11831,14 +12331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:34:49</t>
+          <t>Última actualización: 18:53:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 53</t>
         </is>
       </c>
     </row>
@@ -13072,25 +13572,25 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>18:57</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>103</v>
+        <v>4</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
@@ -13102,18 +13602,93 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>20:17</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>103</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>85</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>20:28</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D55" t="n">
-        <v>114</v>
-      </c>
-      <c r="E55" t="inlineStr">
+      <c r="D57" t="n">
+        <v>95</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>108</v>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4229
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E421"/>
+  <dimension ref="A1:E433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:06</t>
+          <t>Última actualización: 19:10:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 416</t>
+          <t>Total filas: 428</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -3508,7 +3508,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6798,7 +6798,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -6808,11 +6808,11 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -6833,11 +6833,11 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -7998,7 +7998,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -8008,11 +8008,11 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8033,7 +8033,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D308" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D336" t="n">
@@ -8948,7 +8948,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -8958,11 +8958,11 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,7 +8973,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -8983,11 +8983,11 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -9008,11 +9008,11 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9758,7 +9758,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D377" t="n">
@@ -9783,7 +9783,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D378" t="n">
@@ -9848,7 +9848,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
@@ -9858,11 +9858,11 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9873,7 +9873,7 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
@@ -9883,11 +9883,11 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E382" t="inlineStr">
         <is>
@@ -9973,7 +9973,7 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
@@ -9987,7 +9987,7 @@
         </is>
       </c>
       <c r="D386" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E386" t="inlineStr">
         <is>
@@ -9998,21 +9998,21 @@
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="E387" t="inlineStr">
         <is>
@@ -10023,21 +10023,21 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10053,16 +10053,16 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10073,21 +10073,21 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D390" t="n">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="E390" t="inlineStr">
         <is>
@@ -10098,12 +10098,12 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
@@ -10112,7 +10112,7 @@
         </is>
       </c>
       <c r="D391" t="n">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="E391" t="inlineStr">
         <is>
@@ -10123,21 +10123,21 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,21 +10148,21 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>28</v>
+        <v>72</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10173,21 +10173,21 @@
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D394" t="n">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="E394" t="inlineStr">
         <is>
@@ -10203,16 +10203,16 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D395" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="E395" t="inlineStr">
         <is>
@@ -10223,21 +10223,21 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D396" t="n">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="E396" t="inlineStr">
         <is>
@@ -10253,16 +10253,16 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>19:29</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D397" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="E397" t="inlineStr">
         <is>
@@ -10273,21 +10273,21 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="E398" t="inlineStr">
         <is>
@@ -10298,21 +10298,21 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>19:39</t>
+          <t>19:28</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="E399" t="inlineStr">
         <is>
@@ -10323,21 +10323,21 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>19:42</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D400" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -10348,21 +10348,21 @@
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D401" t="n">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="E401" t="inlineStr">
         <is>
@@ -10373,21 +10373,21 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>19:39</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D402" t="n">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="E402" t="inlineStr">
         <is>
@@ -10403,16 +10403,16 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:42</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E403" t="inlineStr">
         <is>
@@ -10423,12 +10423,12 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -10437,7 +10437,7 @@
         </is>
       </c>
       <c r="D404" t="n">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="E404" t="inlineStr">
         <is>
@@ -10448,21 +10448,21 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D405" t="n">
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="E405" t="inlineStr">
         <is>
@@ -10473,21 +10473,21 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D406" t="n">
-        <v>69</v>
+        <v>36</v>
       </c>
       <c r="E406" t="inlineStr">
         <is>
@@ -10498,21 +10498,21 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>91</v>
+        <v>53</v>
       </c>
       <c r="E407" t="inlineStr">
         <is>
@@ -10523,21 +10523,21 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="E408" t="inlineStr">
         <is>
@@ -10548,21 +10548,21 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D409" t="n">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="E409" t="inlineStr">
         <is>
@@ -10573,21 +10573,21 @@
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D410" t="n">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="E410" t="inlineStr">
         <is>
@@ -10598,21 +10598,21 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D411" t="n">
-        <v>82</v>
+        <v>52</v>
       </c>
       <c r="E411" t="inlineStr">
         <is>
@@ -10623,21 +10623,21 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D412" t="n">
-        <v>103</v>
+        <v>55</v>
       </c>
       <c r="E412" t="inlineStr">
         <is>
@@ -10648,21 +10648,21 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>20:18</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D413" t="n">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="E413" t="inlineStr">
         <is>
@@ -10678,16 +10678,16 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>20:18</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D414" t="n">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="E414" t="inlineStr">
         <is>
@@ -10703,16 +10703,16 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>20:21</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D415" t="n">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="E415" t="inlineStr">
         <is>
@@ -10723,21 +10723,21 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D416" t="n">
-        <v>109</v>
+        <v>56</v>
       </c>
       <c r="E416" t="inlineStr">
         <is>
@@ -10748,21 +10748,21 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:13</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D417" t="n">
-        <v>109</v>
+        <v>63</v>
       </c>
       <c r="E417" t="inlineStr">
         <is>
@@ -10778,16 +10778,16 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>20:28</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D418" t="n">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="E418" t="inlineStr">
         <is>
@@ -10798,21 +10798,21 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>20:33</t>
+          <t>20:17</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E419" t="inlineStr">
         <is>
@@ -10828,16 +10828,16 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:18</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D420" t="n">
-        <v>109</v>
+        <v>85</v>
       </c>
       <c r="E420" t="inlineStr">
         <is>
@@ -10848,23 +10848,323 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
+          <t>19:10:39</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>68</v>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>19:10:39</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D422" t="n">
+        <v>70</v>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
           <t>18:53:06</t>
         </is>
       </c>
-      <c r="B421" t="inlineStr">
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>20:21</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>88</v>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>109</v>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>18:34:49</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>109</v>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>19:10:39</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>20:28</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>78</v>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>19:10:39</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>20:32</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>82</v>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>20:33</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>100</v>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>19:10:39</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>91</v>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>109</v>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>19:10:39</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>20:47</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>97</v>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
         <is>
           <t>20:48</t>
         </is>
       </c>
-      <c r="C421" t="inlineStr">
+      <c r="C432" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D421" t="n">
+      <c r="D432" t="n">
         <v>115</v>
       </c>
-      <c r="E421" t="inlineStr">
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>19:10:39</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>20:53</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>103</v>
+      </c>
+      <c r="E433" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10881,7 +11181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10894,14 +11194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:06</t>
+          <t>Última actualización: 19:10:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 55</t>
+          <t>Total filas: 58</t>
         </is>
       </c>
     </row>
@@ -12210,7 +12510,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -12224,7 +12524,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -12235,12 +12535,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>20:33</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -12249,7 +12549,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -12265,16 +12565,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:33</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -12285,23 +12585,98 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>19:10:39</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>91</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>18:53:06</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>109</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>19:10:39</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>20:47</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>97</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
         <is>
           <t>20:48</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D60" t="n">
+      <c r="D63" t="n">
         <v>115</v>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -12318,7 +12693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12331,14 +12706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:06</t>
+          <t>Última actualización: 19:10:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 53</t>
+          <t>Total filas: 54</t>
         </is>
       </c>
     </row>
@@ -13597,7 +13972,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -13611,7 +13986,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -13647,7 +14022,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -13661,7 +14036,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -13672,7 +14047,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -13686,11 +14061,36 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>19:10:39</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>117</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4230
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E433"/>
+  <dimension ref="A1:E446"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:10:39</t>
+          <t>Última actualización: 19:40:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 428</t>
+          <t>Total filas: 441</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>59</v>
+        <v>97</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>9</v>
+        <v>119</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -6183,7 +6183,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6798,7 +6798,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -6808,11 +6808,11 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -6833,11 +6833,11 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -7273,7 +7273,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -7283,11 +7283,11 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7308,11 +7308,11 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D297" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7998,7 +7998,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -8008,11 +8008,11 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8773,7 +8773,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -8783,11 +8783,11 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,7 +8798,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -8808,11 +8808,11 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8883,7 +8883,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D342" t="n">
@@ -8908,7 +8908,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D343" t="n">
@@ -8948,7 +8948,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -8958,11 +8958,11 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,7 +8973,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -8983,11 +8983,11 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -9008,11 +9008,11 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9333,7 +9333,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D360" t="n">
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9848,7 +9848,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
@@ -9858,11 +9858,11 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9873,7 +9873,7 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
@@ -9883,11 +9883,11 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="E382" t="inlineStr">
         <is>
@@ -10398,21 +10398,21 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>19:42</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E403" t="inlineStr">
         <is>
@@ -10423,21 +10423,21 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>19:42</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D404" t="n">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="E404" t="inlineStr">
         <is>
@@ -10448,7 +10448,7 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
@@ -10462,7 +10462,7 @@
         </is>
       </c>
       <c r="D405" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="E405" t="inlineStr">
         <is>
@@ -10473,12 +10473,12 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -10487,7 +10487,7 @@
         </is>
       </c>
       <c r="D406" t="n">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="E406" t="inlineStr">
         <is>
@@ -10498,7 +10498,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -10508,11 +10508,11 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="E407" t="inlineStr">
         <is>
@@ -10523,21 +10523,21 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="E408" t="inlineStr">
         <is>
@@ -10548,21 +10548,21 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>19:59</t>
+          <t>19:52</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D409" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E409" t="inlineStr">
         <is>
@@ -10573,21 +10573,21 @@
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D410" t="n">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="E410" t="inlineStr">
         <is>
@@ -10598,21 +10598,21 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D411" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="E411" t="inlineStr">
         <is>
@@ -10628,7 +10628,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -10637,7 +10637,7 @@
         </is>
       </c>
       <c r="D412" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E412" t="inlineStr">
         <is>
@@ -10648,21 +10648,21 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D413" t="n">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E413" t="inlineStr">
         <is>
@@ -10673,21 +10673,21 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D414" t="n">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="E414" t="inlineStr">
         <is>
@@ -10698,21 +10698,21 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D415" t="n">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="E415" t="inlineStr">
         <is>
@@ -10723,21 +10723,21 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D416" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="E416" t="inlineStr">
         <is>
@@ -10748,21 +10748,21 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>20:13</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D417" t="n">
-        <v>63</v>
+        <v>26</v>
       </c>
       <c r="E417" t="inlineStr">
         <is>
@@ -10778,16 +10778,16 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D418" t="n">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="E418" t="inlineStr">
         <is>
@@ -10798,21 +10798,21 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E419" t="inlineStr">
         <is>
@@ -10823,21 +10823,21 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>20:18</t>
+          <t>20:13</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D420" t="n">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="E420" t="inlineStr">
         <is>
@@ -10848,21 +10848,21 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>20:18</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D421" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="E421" t="inlineStr">
         <is>
@@ -10873,21 +10873,21 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D422" t="n">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="E422" t="inlineStr">
         <is>
@@ -10898,21 +10898,21 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>20:21</t>
+          <t>20:17</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D423" t="n">
-        <v>88</v>
+        <v>37</v>
       </c>
       <c r="E423" t="inlineStr">
         <is>
@@ -10923,21 +10923,21 @@
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:17</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D424" t="n">
-        <v>109</v>
+        <v>37</v>
       </c>
       <c r="E424" t="inlineStr">
         <is>
@@ -10948,21 +10948,21 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:18</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D425" t="n">
-        <v>109</v>
+        <v>68</v>
       </c>
       <c r="E425" t="inlineStr">
         <is>
@@ -10973,21 +10973,21 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>20:28</t>
+          <t>20:18</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D426" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E426" t="inlineStr">
         <is>
@@ -10998,21 +10998,21 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:20</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D427" t="n">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="E427" t="inlineStr">
         <is>
@@ -11028,16 +11028,16 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>20:33</t>
+          <t>20:21</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D428" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="E428" t="inlineStr">
         <is>
@@ -11048,21 +11048,21 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D429" t="n">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="E429" t="inlineStr">
         <is>
@@ -11073,17 +11073,17 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D430" t="n">
@@ -11098,21 +11098,21 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>20:47</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D431" t="n">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="E431" t="inlineStr">
         <is>
@@ -11123,21 +11123,21 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>20:48</t>
+          <t>20:28</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D432" t="n">
-        <v>115</v>
+        <v>78</v>
       </c>
       <c r="E432" t="inlineStr">
         <is>
@@ -11148,23 +11148,348 @@
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
+          <t>20:32</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>52</v>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>20:33</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D434" t="n">
+        <v>100</v>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>19:40:57</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D435" t="n">
+        <v>61</v>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D436" t="n">
+        <v>109</v>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>19:40:57</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>20:47</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D437" t="n">
+        <v>67</v>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>18:53:06</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>20:48</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D438" t="n">
+        <v>115</v>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>19:40:57</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
           <t>20:53</t>
         </is>
       </c>
-      <c r="C433" t="inlineStr">
+      <c r="C439" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D433" t="n">
-        <v>103</v>
-      </c>
-      <c r="E433" t="inlineStr">
+      <c r="D439" t="n">
+        <v>73</v>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>19:40:57</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D440" t="n">
+        <v>76</v>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>19:40:57</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D441" t="n">
+        <v>85</v>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>19:40:57</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>21:12</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D442" t="n">
+        <v>92</v>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>19:40:57</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>21:19</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D443" t="n">
+        <v>99</v>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>19:40:57</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>21:20</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D444" t="n">
+        <v>100</v>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>19:40:57</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D445" t="n">
+        <v>112</v>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>19:40:57</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D446" t="n">
+        <v>115</v>
+      </c>
+      <c r="E446" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11194,7 +11519,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:10:39</t>
+          <t>Última actualización: 19:40:57</t>
         </is>
       </c>
     </row>
@@ -11570,7 +11895,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -11595,7 +11920,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -12535,7 +12860,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -12549,7 +12874,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>82</v>
+        <v>52</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -12585,7 +12910,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -12599,7 +12924,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -12635,7 +12960,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -12649,7 +12974,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>97</v>
+        <v>67</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -12706,7 +13031,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:10:39</t>
+          <t>Última actualización: 19:40:57</t>
         </is>
       </c>
     </row>
@@ -13972,7 +14297,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -13986,7 +14311,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -14022,7 +14347,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -14036,7 +14361,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -14047,7 +14372,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -14061,7 +14386,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -14072,7 +14397,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -14086,7 +14411,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4231
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E446"/>
+  <dimension ref="A1:E450"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:40:57</t>
+          <t>Última actualización: 19:59:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 441</t>
+          <t>Total filas: 445</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>9</v>
+        <v>119</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -6183,7 +6183,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D297" t="n">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -8123,7 +8123,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -8133,11 +8133,11 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,7 +8148,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -8158,11 +8158,11 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8173,7 +8173,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -8183,11 +8183,11 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,7 +8198,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -8208,11 +8208,11 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D336" t="n">
@@ -8773,7 +8773,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -8783,11 +8783,11 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,7 +8798,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -8808,11 +8808,11 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8948,7 +8948,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -8958,11 +8958,11 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,7 +8973,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -8983,11 +8983,11 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -9008,11 +9008,11 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9758,7 +9758,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D377" t="n">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D379" t="n">
@@ -10458,7 +10458,7 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D405" t="n">
@@ -10483,7 +10483,7 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D406" t="n">
@@ -10498,7 +10498,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -10508,11 +10508,11 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="E407" t="inlineStr">
         <is>
@@ -10523,7 +10523,7 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
@@ -10533,11 +10533,11 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="E408" t="inlineStr">
         <is>
@@ -10648,12 +10648,12 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -10662,7 +10662,7 @@
         </is>
       </c>
       <c r="D413" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="E413" t="inlineStr">
         <is>
@@ -10673,21 +10673,21 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D414" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E414" t="inlineStr">
         <is>
@@ -10703,16 +10703,16 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D415" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E415" t="inlineStr">
         <is>
@@ -10723,21 +10723,21 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D416" t="n">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="E416" t="inlineStr">
         <is>
@@ -10748,21 +10748,21 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D417" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E417" t="inlineStr">
         <is>
@@ -10773,21 +10773,21 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D418" t="n">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="E418" t="inlineStr">
         <is>
@@ -10808,7 +10808,7 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D419" t="n">
@@ -10823,21 +10823,21 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>20:13</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D420" t="n">
-        <v>33</v>
+        <v>73</v>
       </c>
       <c r="E420" t="inlineStr">
         <is>
@@ -10848,21 +10848,21 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D421" t="n">
-        <v>82</v>
+        <v>7</v>
       </c>
       <c r="E421" t="inlineStr">
         <is>
@@ -10873,21 +10873,21 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:13</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D422" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="E422" t="inlineStr">
         <is>
@@ -10898,21 +10898,21 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D423" t="n">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="E423" t="inlineStr">
         <is>
@@ -10923,21 +10923,21 @@
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D424" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="E424" t="inlineStr">
         <is>
@@ -10948,12 +10948,12 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>20:18</t>
+          <t>20:17</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -10962,7 +10962,7 @@
         </is>
       </c>
       <c r="D425" t="n">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="E425" t="inlineStr">
         <is>
@@ -10973,12 +10973,12 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>20:18</t>
+          <t>20:17</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -10987,7 +10987,7 @@
         </is>
       </c>
       <c r="D426" t="n">
-        <v>85</v>
+        <v>18</v>
       </c>
       <c r="E426" t="inlineStr">
         <is>
@@ -10998,21 +10998,21 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>20:18</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D427" t="n">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="E427" t="inlineStr">
         <is>
@@ -11028,16 +11028,16 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>20:21</t>
+          <t>20:18</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D428" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E428" t="inlineStr">
         <is>
@@ -11048,21 +11048,21 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:20</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D429" t="n">
-        <v>109</v>
+        <v>21</v>
       </c>
       <c r="E429" t="inlineStr">
         <is>
@@ -11073,12 +11073,12 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:21</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
@@ -11087,7 +11087,7 @@
         </is>
       </c>
       <c r="D430" t="n">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="E430" t="inlineStr">
         <is>
@@ -11098,21 +11098,21 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D431" t="n">
-        <v>47</v>
+        <v>109</v>
       </c>
       <c r="E431" t="inlineStr">
         <is>
@@ -11123,21 +11123,21 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>20:28</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D432" t="n">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="E432" t="inlineStr">
         <is>
@@ -11153,16 +11153,16 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D433" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E433" t="inlineStr">
         <is>
@@ -11173,21 +11173,21 @@
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>20:33</t>
+          <t>20:28</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D434" t="n">
-        <v>100</v>
+        <v>29</v>
       </c>
       <c r="E434" t="inlineStr">
         <is>
@@ -11198,21 +11198,21 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="E435" t="inlineStr">
         <is>
@@ -11228,16 +11228,16 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:33</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D436" t="n">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="E436" t="inlineStr">
         <is>
@@ -11248,21 +11248,21 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>20:47</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D437" t="n">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="E437" t="inlineStr">
         <is>
@@ -11278,16 +11278,16 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>20:48</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D438" t="n">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E438" t="inlineStr">
         <is>
@@ -11298,21 +11298,21 @@
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:47</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D439" t="n">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="E439" t="inlineStr">
         <is>
@@ -11323,21 +11323,21 @@
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:48</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D440" t="n">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="E440" t="inlineStr">
         <is>
@@ -11348,21 +11348,21 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D441" t="n">
-        <v>85</v>
+        <v>51</v>
       </c>
       <c r="E441" t="inlineStr">
         <is>
@@ -11373,21 +11373,21 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>21:12</t>
+          <t>20:53</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D442" t="n">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="E442" t="inlineStr">
         <is>
@@ -11398,21 +11398,21 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>21:19</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D443" t="n">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="E443" t="inlineStr">
         <is>
@@ -11423,21 +11423,21 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>21:20</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D444" t="n">
-        <v>100</v>
+        <v>66</v>
       </c>
       <c r="E444" t="inlineStr">
         <is>
@@ -11448,21 +11448,21 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>21:32</t>
+          <t>21:12</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D445" t="n">
-        <v>112</v>
+        <v>73</v>
       </c>
       <c r="E445" t="inlineStr">
         <is>
@@ -11473,23 +11473,123 @@
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
+          <t>21:19</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D446" t="n">
+        <v>80</v>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>19:59:51</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>21:20</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D447" t="n">
+        <v>81</v>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>19:59:51</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D448" t="n">
+        <v>93</v>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>19:59:51</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C446" t="inlineStr">
+      <c r="C449" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D446" t="n">
-        <v>115</v>
-      </c>
-      <c r="E446" t="inlineStr">
+      <c r="D449" t="n">
+        <v>96</v>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>19:59:51</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>21:51</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D450" t="n">
+        <v>112</v>
+      </c>
+      <c r="E450" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11519,7 +11619,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:40:57</t>
+          <t>Última actualización: 19:59:51</t>
         </is>
       </c>
     </row>
@@ -11895,7 +11995,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -11920,7 +12020,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -12860,7 +12960,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -12874,7 +12974,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -12910,7 +13010,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -12924,7 +13024,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -12960,7 +13060,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -12974,7 +13074,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -13031,7 +13131,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:40:57</t>
+          <t>Última actualización: 19:59:51</t>
         </is>
       </c>
     </row>
@@ -14297,7 +14397,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -14311,7 +14411,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -14347,7 +14447,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -14361,7 +14461,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -14372,7 +14472,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -14386,7 +14486,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -14397,7 +14497,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -14411,7 +14511,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4232
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E450"/>
+  <dimension ref="A1:E462"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:59:51</t>
+          <t>Última actualización: 20:21:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 445</t>
+          <t>Total filas: 457</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -6183,7 +6183,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6758,7 +6758,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
@@ -6783,7 +6783,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7273,7 +7273,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -7283,11 +7283,11 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7308,11 +7308,11 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7983,11 +7983,11 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,7 +7998,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -8008,11 +8008,11 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,7 +8023,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -8033,11 +8033,11 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D336" t="n">
@@ -8773,7 +8773,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -8783,11 +8783,11 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,7 +8798,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -8808,11 +8808,11 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8883,7 +8883,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D342" t="n">
@@ -8908,7 +8908,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D343" t="n">
@@ -8948,7 +8948,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -8958,11 +8958,11 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,7 +8973,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -8983,11 +8983,11 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,7 +9098,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -9108,11 +9108,11 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9333,7 +9333,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D360" t="n">
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9848,7 +9848,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
@@ -9858,11 +9858,11 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9873,7 +9873,7 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
@@ -9883,11 +9883,11 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E382" t="inlineStr">
         <is>
@@ -10498,7 +10498,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -10508,11 +10508,11 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="E407" t="inlineStr">
         <is>
@@ -10523,7 +10523,7 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
@@ -10533,11 +10533,11 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="E408" t="inlineStr">
         <is>
@@ -10658,7 +10658,7 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D413" t="n">
@@ -10683,7 +10683,7 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D414" t="n">
@@ -10798,7 +10798,7 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
@@ -10808,11 +10808,11 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>73</v>
+        <v>7</v>
       </c>
       <c r="E419" t="inlineStr">
         <is>
@@ -10848,7 +10848,7 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
@@ -10858,11 +10858,11 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D421" t="n">
-        <v>7</v>
+        <v>73</v>
       </c>
       <c r="E421" t="inlineStr">
         <is>
@@ -10958,7 +10958,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D425" t="n">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D426" t="n">
@@ -11073,7 +11073,7 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
@@ -11087,7 +11087,7 @@
         </is>
       </c>
       <c r="D430" t="n">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="E430" t="inlineStr">
         <is>
@@ -11173,7 +11173,7 @@
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
@@ -11187,7 +11187,7 @@
         </is>
       </c>
       <c r="D434" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="E434" t="inlineStr">
         <is>
@@ -11223,7 +11223,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -11237,7 +11237,7 @@
         </is>
       </c>
       <c r="D436" t="n">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="E436" t="inlineStr">
         <is>
@@ -11248,7 +11248,7 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
@@ -11262,7 +11262,7 @@
         </is>
       </c>
       <c r="D437" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="E437" t="inlineStr">
         <is>
@@ -11298,7 +11298,7 @@
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
@@ -11312,7 +11312,7 @@
         </is>
       </c>
       <c r="D439" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E439" t="inlineStr">
         <is>
@@ -11348,7 +11348,7 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
@@ -11362,7 +11362,7 @@
         </is>
       </c>
       <c r="D441" t="n">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="E441" t="inlineStr">
         <is>
@@ -11373,21 +11373,21 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D442" t="n">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="E442" t="inlineStr">
         <is>
@@ -11398,21 +11398,21 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:53</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D443" t="n">
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="E443" t="inlineStr">
         <is>
@@ -11423,21 +11423,21 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D444" t="n">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="E444" t="inlineStr">
         <is>
@@ -11453,16 +11453,16 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>21:12</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D445" t="n">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="E445" t="inlineStr">
         <is>
@@ -11473,21 +11473,21 @@
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>21:19</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D446" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="E446" t="inlineStr">
         <is>
@@ -11503,16 +11503,16 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>21:20</t>
+          <t>21:12</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D447" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E447" t="inlineStr">
         <is>
@@ -11523,21 +11523,21 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>21:32</t>
+          <t>21:13</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D448" t="n">
-        <v>93</v>
+        <v>52</v>
       </c>
       <c r="E448" t="inlineStr">
         <is>
@@ -11548,21 +11548,21 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:18</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D449" t="n">
-        <v>96</v>
+        <v>57</v>
       </c>
       <c r="E449" t="inlineStr">
         <is>
@@ -11578,18 +11578,318 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
+          <t>21:19</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D450" t="n">
+        <v>80</v>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>19:59:51</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>21:20</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D451" t="n">
+        <v>81</v>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>20:21:24</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>21:20</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D452" t="n">
+        <v>59</v>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>20:21:24</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>21:21</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D453" t="n">
+        <v>60</v>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>20:21:24</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D454" t="n">
+        <v>69</v>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>19:59:51</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D455" t="n">
+        <v>93</v>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>20:21:24</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>21:33</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D456" t="n">
+        <v>72</v>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>19:59:51</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D457" t="n">
+        <v>96</v>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>20:21:24</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D458" t="n">
+        <v>75</v>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>19:59:51</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
           <t>21:51</t>
         </is>
       </c>
-      <c r="C450" t="inlineStr">
+      <c r="C459" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D450" t="n">
+      <c r="D459" t="n">
         <v>112</v>
       </c>
-      <c r="E450" t="inlineStr">
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>20:21:24</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D460" t="n">
+        <v>91</v>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>20:21:24</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>22:01</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D461" t="n">
+        <v>100</v>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>20:21:24</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D462" t="n">
+        <v>107</v>
+      </c>
+      <c r="E462" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11619,7 +11919,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:59:51</t>
+          <t>Última actualización: 20:21:24</t>
         </is>
       </c>
     </row>
@@ -11995,7 +12295,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -12020,7 +12320,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -12985,7 +13285,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -12999,7 +13299,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -13010,7 +13310,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -13024,7 +13324,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -13060,7 +13360,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -13074,7 +13374,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -13118,7 +13418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13131,14 +13431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:59:51</t>
+          <t>Última actualización: 20:21:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 54</t>
+          <t>Total filas: 57</t>
         </is>
       </c>
     </row>
@@ -14447,46 +14747,46 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>20:28</t>
+          <t>20:21</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:28</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>42</v>
+        <v>7</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -14497,25 +14797,100 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>20:21:24</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>20</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>19:59:51</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>21:07</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D60" t="n">
         <v>68</v>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>20:21:24</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>21:08</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>47</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>20:21:24</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>111</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4233
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E462"/>
+  <dimension ref="A1:E470"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:21:24</t>
+          <t>Última actualización: 20:43:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 457</t>
+          <t>Total filas: 465</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6798,7 +6798,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>14:11:32</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -6808,11 +6808,11 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>14:11:32</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -6833,11 +6833,11 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D297" t="n">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7983,11 +7983,11 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,7 +7998,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -8008,11 +8008,11 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,7 +8023,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -8033,11 +8033,11 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8173,7 +8173,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -8183,11 +8183,11 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,7 +8198,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -8208,11 +8208,11 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8648,7 +8648,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -8658,11 +8658,11 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,7 +8673,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -8683,11 +8683,11 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8773,7 +8773,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -8783,11 +8783,11 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,7 +8798,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -8808,11 +8808,11 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8973,7 +8973,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -8983,11 +8983,11 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -9008,11 +9008,11 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,7 +9098,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -9108,11 +9108,11 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9333,7 +9333,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D360" t="n">
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9758,7 +9758,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D377" t="n">
@@ -9783,7 +9783,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D378" t="n">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D379" t="n">
@@ -9848,7 +9848,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
@@ -9858,11 +9858,11 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9873,7 +9873,7 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
@@ -9883,11 +9883,11 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="E382" t="inlineStr">
         <is>
@@ -10458,7 +10458,7 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D405" t="n">
@@ -10483,7 +10483,7 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D406" t="n">
@@ -10498,7 +10498,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -10508,11 +10508,11 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="E407" t="inlineStr">
         <is>
@@ -10523,7 +10523,7 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
@@ -10533,11 +10533,11 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="E408" t="inlineStr">
         <is>
@@ -10623,7 +10623,7 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
@@ -10633,11 +10633,11 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D412" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E412" t="inlineStr">
         <is>
@@ -10673,7 +10673,7 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
@@ -10683,11 +10683,11 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D414" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E414" t="inlineStr">
         <is>
@@ -10748,7 +10748,7 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
@@ -10758,11 +10758,11 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D417" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="E417" t="inlineStr">
         <is>
@@ -10773,7 +10773,7 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
@@ -10783,11 +10783,11 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D418" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="E418" t="inlineStr">
         <is>
@@ -10958,7 +10958,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D425" t="n">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D426" t="n">
@@ -11323,7 +11323,7 @@
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
@@ -11337,7 +11337,7 @@
         </is>
       </c>
       <c r="D440" t="n">
-        <v>115</v>
+        <v>5</v>
       </c>
       <c r="E440" t="inlineStr">
         <is>
@@ -11373,21 +11373,21 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>20:52</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D442" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="E442" t="inlineStr">
         <is>
@@ -11398,21 +11398,21 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D443" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E443" t="inlineStr">
         <is>
@@ -11428,16 +11428,16 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:53</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D444" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E444" t="inlineStr">
         <is>
@@ -11448,21 +11448,21 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:54</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D445" t="n">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="E445" t="inlineStr">
         <is>
@@ -11478,16 +11478,16 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D446" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E446" t="inlineStr">
         <is>
@@ -11498,21 +11498,21 @@
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>21:12</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D447" t="n">
-        <v>73</v>
+        <v>14</v>
       </c>
       <c r="E447" t="inlineStr">
         <is>
@@ -11523,21 +11523,21 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>21:13</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D448" t="n">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="E448" t="inlineStr">
         <is>
@@ -11548,21 +11548,21 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>21:18</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D449" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="E449" t="inlineStr">
         <is>
@@ -11578,16 +11578,16 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>21:19</t>
+          <t>21:12</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D450" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E450" t="inlineStr">
         <is>
@@ -11598,21 +11598,21 @@
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>21:20</t>
+          <t>21:13</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D451" t="n">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="E451" t="inlineStr">
         <is>
@@ -11623,21 +11623,21 @@
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>21:20</t>
+          <t>21:18</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D452" t="n">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="E452" t="inlineStr">
         <is>
@@ -11648,21 +11648,21 @@
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>21:21</t>
+          <t>21:19</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D453" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="E453" t="inlineStr">
         <is>
@@ -11673,21 +11673,21 @@
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:20</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D454" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="E454" t="inlineStr">
         <is>
@@ -11698,21 +11698,21 @@
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>21:32</t>
+          <t>21:20</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D455" t="n">
-        <v>93</v>
+        <v>37</v>
       </c>
       <c r="E455" t="inlineStr">
         <is>
@@ -11723,21 +11723,21 @@
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>21:33</t>
+          <t>21:21</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D456" t="n">
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="E456" t="inlineStr">
         <is>
@@ -11748,21 +11748,21 @@
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:21:24</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D457" t="n">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="E457" t="inlineStr">
         <is>
@@ -11773,21 +11773,21 @@
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:31</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D458" t="n">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="E458" t="inlineStr">
         <is>
@@ -11803,16 +11803,16 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>21:51</t>
+          <t>21:32</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D459" t="n">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="E459" t="inlineStr">
         <is>
@@ -11823,21 +11823,21 @@
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>21:52</t>
+          <t>21:33</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D460" t="n">
-        <v>91</v>
+        <v>50</v>
       </c>
       <c r="E460" t="inlineStr">
         <is>
@@ -11848,21 +11848,21 @@
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>22:01</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D461" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E461" t="inlineStr">
         <is>
@@ -11873,23 +11873,223 @@
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D462" t="n">
+        <v>53</v>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>19:59:51</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>21:51</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D463" t="n">
+        <v>112</v>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D464" t="n">
+        <v>69</v>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>22:01</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D465" t="n">
+        <v>78</v>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
           <t>20:21:24</t>
         </is>
       </c>
-      <c r="B462" t="inlineStr">
+      <c r="B466" t="inlineStr">
         <is>
           <t>22:08</t>
         </is>
       </c>
-      <c r="C462" t="inlineStr">
+      <c r="C466" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D462" t="n">
+      <c r="D466" t="n">
         <v>107</v>
       </c>
-      <c r="E462" t="inlineStr">
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D467" t="n">
+        <v>86</v>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D468" t="n">
+        <v>98</v>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>22:32</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D469" t="n">
+        <v>109</v>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>22:39</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D470" t="n">
+        <v>116</v>
+      </c>
+      <c r="E470" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11919,7 +12119,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:21:24</t>
+          <t>Última actualización: 20:43:05</t>
         </is>
       </c>
     </row>
@@ -13385,7 +13585,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -13399,7 +13599,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>115</v>
+        <v>5</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -13418,7 +13618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13431,14 +13631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:21:24</t>
+          <t>Última actualización: 20:43:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 57</t>
+          <t>Total filas: 59</t>
         </is>
       </c>
     </row>
@@ -14847,7 +15047,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -14861,7 +15061,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -14872,23 +15072,73 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>75</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
           <t>22:12</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D62" t="n">
-        <v>111</v>
-      </c>
-      <c r="E62" t="inlineStr">
+      <c r="D63" t="n">
+        <v>89</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>98</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4234
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E470"/>
+  <dimension ref="A1:E477"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:43:05</t>
+          <t>Última actualización: 20:59:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 465</t>
+          <t>Total filas: 472</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>04:55:30</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:55:30</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1108,11 +1108,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -7273,7 +7273,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>15:06:33</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -7283,11 +7283,11 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>15:06:33</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7308,11 +7308,11 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -7998,7 +7998,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -8008,11 +8008,11 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8033,7 +8033,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D308" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8173,7 +8173,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -8183,11 +8183,11 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,7 +8198,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -8208,11 +8208,11 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8648,7 +8648,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -8658,11 +8658,11 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,7 +8673,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -8683,11 +8683,11 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8883,7 +8883,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D342" t="n">
@@ -8908,7 +8908,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D343" t="n">
@@ -8973,7 +8973,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -8983,11 +8983,11 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -9008,11 +9008,11 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9333,7 +9333,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D360" t="n">
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9758,7 +9758,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D377" t="n">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D379" t="n">
@@ -10123,7 +10123,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -10133,11 +10133,11 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,7 +10148,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -10158,11 +10158,11 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>72</v>
+        <v>8</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10458,7 +10458,7 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D405" t="n">
@@ -10483,7 +10483,7 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D406" t="n">
@@ -10623,7 +10623,7 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
@@ -10633,11 +10633,11 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D412" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E412" t="inlineStr">
         <is>
@@ -10673,7 +10673,7 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
@@ -10683,11 +10683,11 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D414" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E414" t="inlineStr">
         <is>
@@ -10958,7 +10958,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D425" t="n">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D426" t="n">
@@ -11108,7 +11108,7 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D431" t="n">
@@ -11133,7 +11133,7 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D432" t="n">
@@ -11548,7 +11548,7 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
@@ -11562,7 +11562,7 @@
         </is>
       </c>
       <c r="D449" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="E449" t="inlineStr">
         <is>
@@ -11573,7 +11573,7 @@
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
@@ -11587,7 +11587,7 @@
         </is>
       </c>
       <c r="D450" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E450" t="inlineStr">
         <is>
@@ -11623,7 +11623,7 @@
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
@@ -11637,7 +11637,7 @@
         </is>
       </c>
       <c r="D452" t="n">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="E452" t="inlineStr">
         <is>
@@ -11648,7 +11648,7 @@
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
@@ -11662,7 +11662,7 @@
         </is>
       </c>
       <c r="D453" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="E453" t="inlineStr">
         <is>
@@ -11673,7 +11673,7 @@
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
@@ -11683,11 +11683,11 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D454" t="n">
-        <v>81</v>
+        <v>37</v>
       </c>
       <c r="E454" t="inlineStr">
         <is>
@@ -11698,7 +11698,7 @@
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
@@ -11708,11 +11708,11 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D455" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E455" t="inlineStr">
         <is>
@@ -11748,7 +11748,7 @@
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
@@ -11762,7 +11762,7 @@
         </is>
       </c>
       <c r="D457" t="n">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="E457" t="inlineStr">
         <is>
@@ -11798,7 +11798,7 @@
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
@@ -11812,7 +11812,7 @@
         </is>
       </c>
       <c r="D459" t="n">
-        <v>93</v>
+        <v>33</v>
       </c>
       <c r="E459" t="inlineStr">
         <is>
@@ -11873,7 +11873,7 @@
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
@@ -11887,7 +11887,7 @@
         </is>
       </c>
       <c r="D462" t="n">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="E462" t="inlineStr">
         <is>
@@ -11898,21 +11898,21 @@
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>21:51</t>
+          <t>21:46</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D463" t="n">
-        <v>112</v>
+        <v>47</v>
       </c>
       <c r="E463" t="inlineStr">
         <is>
@@ -11923,12 +11923,12 @@
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>21:52</t>
+          <t>21:51</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
@@ -11937,7 +11937,7 @@
         </is>
       </c>
       <c r="D464" t="n">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="E464" t="inlineStr">
         <is>
@@ -11953,16 +11953,16 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>22:01</t>
+          <t>21:52</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D465" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E465" t="inlineStr">
         <is>
@@ -11973,21 +11973,21 @@
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>20:21:24</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>22:08</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D466" t="n">
-        <v>107</v>
+        <v>61</v>
       </c>
       <c r="E466" t="inlineStr">
         <is>
@@ -12003,16 +12003,16 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>22:09</t>
+          <t>22:01</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D467" t="n">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E467" t="inlineStr">
         <is>
@@ -12023,21 +12023,21 @@
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>22:21</t>
+          <t>22:08</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D468" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="E468" t="inlineStr">
         <is>
@@ -12053,16 +12053,16 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>22:32</t>
+          <t>22:09</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D469" t="n">
-        <v>109</v>
+        <v>86</v>
       </c>
       <c r="E469" t="inlineStr">
         <is>
@@ -12073,23 +12073,198 @@
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
+          <t>20:59:36</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>22:20</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D470" t="n">
+        <v>81</v>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
           <t>20:43:05</t>
         </is>
       </c>
-      <c r="B470" t="inlineStr">
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D471" t="n">
+        <v>98</v>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>20:59:36</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>22:24</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D472" t="n">
+        <v>85</v>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>20:59:36</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>22:31</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D473" t="n">
+        <v>92</v>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>22:32</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D474" t="n">
+        <v>109</v>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>20:59:36</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>22:38</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D475" t="n">
+        <v>99</v>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
         <is>
           <t>22:39</t>
         </is>
       </c>
-      <c r="C470" t="inlineStr">
+      <c r="C476" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D470" t="n">
+      <c r="D476" t="n">
         <v>116</v>
       </c>
-      <c r="E470" t="inlineStr">
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>20:59:36</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>22:57</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D477" t="n">
+        <v>118</v>
+      </c>
+      <c r="E477" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -12106,7 +12281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12119,14 +12294,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:43:05</t>
+          <t>Última actualización: 20:59:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 58</t>
+          <t>Total filas: 59</t>
         </is>
       </c>
     </row>
@@ -13602,6 +13777,31 @@
         <v>5</v>
       </c>
       <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>20:59:36</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>22:57</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>118</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -13618,7 +13818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13631,14 +13831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:43:05</t>
+          <t>Última actualización: 20:59:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 59</t>
+          <t>Total filas: 60</t>
         </is>
       </c>
     </row>
@@ -15022,7 +15222,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -15036,7 +15236,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -15072,12 +15272,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>21:58</t>
+          <t>21:57</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -15086,7 +15286,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -15102,43 +15302,68 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>22:12</t>
+          <t>21:58</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>73</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>20:59:36</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
           <t>22:21</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D64" t="n">
-        <v>98</v>
-      </c>
-      <c r="E64" t="inlineStr">
+      <c r="D65" t="n">
+        <v>82</v>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4235
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E477"/>
+  <dimension ref="A1:E488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:59:36</t>
+          <t>Última actualización: 22:11:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 472</t>
+          <t>Total filas: 483</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:29:16</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>08:29:16</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>59</v>
+        <v>97</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D297" t="n">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8123,7 +8123,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -8133,11 +8133,11 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,7 +8148,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -8158,11 +8158,11 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8648,7 +8648,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -8658,11 +8658,11 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,7 +8673,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -8683,11 +8683,11 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D336" t="n">
@@ -8948,7 +8948,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -8958,11 +8958,11 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -9008,11 +9008,11 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9758,7 +9758,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D377" t="n">
@@ -9783,7 +9783,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D378" t="n">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D379" t="n">
@@ -10123,7 +10123,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -10133,11 +10133,11 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>72</v>
+        <v>8</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,7 +10148,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -10158,11 +10158,11 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10498,7 +10498,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -10508,11 +10508,11 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="E407" t="inlineStr">
         <is>
@@ -10523,7 +10523,7 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
@@ -10533,11 +10533,11 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="E408" t="inlineStr">
         <is>
@@ -10623,7 +10623,7 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
@@ -10633,11 +10633,11 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D412" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E412" t="inlineStr">
         <is>
@@ -10648,7 +10648,7 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
@@ -10658,11 +10658,11 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D413" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E413" t="inlineStr">
         <is>
@@ -10798,7 +10798,7 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
@@ -10808,11 +10808,11 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>7</v>
+        <v>73</v>
       </c>
       <c r="E419" t="inlineStr">
         <is>
@@ -10823,7 +10823,7 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
@@ -10833,11 +10833,11 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D420" t="n">
-        <v>73</v>
+        <v>7</v>
       </c>
       <c r="E420" t="inlineStr">
         <is>
@@ -10858,7 +10858,7 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D421" t="n">
@@ -11108,7 +11108,7 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D431" t="n">
@@ -11133,7 +11133,7 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D432" t="n">
@@ -12073,21 +12073,21 @@
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>20:59:36</t>
+          <t>22:11:55</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>22:20</t>
+          <t>22:12</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D470" t="n">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="E470" t="inlineStr">
         <is>
@@ -12098,12 +12098,12 @@
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>22:11:55</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>22:21</t>
+          <t>22:20</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
@@ -12112,7 +12112,7 @@
         </is>
       </c>
       <c r="D471" t="n">
-        <v>98</v>
+        <v>9</v>
       </c>
       <c r="E471" t="inlineStr">
         <is>
@@ -12123,12 +12123,12 @@
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>20:59:36</t>
+          <t>22:11:55</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>22:24</t>
+          <t>22:20</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
@@ -12137,7 +12137,7 @@
         </is>
       </c>
       <c r="D472" t="n">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="E472" t="inlineStr">
         <is>
@@ -12148,21 +12148,21 @@
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>20:59:36</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>22:31</t>
+          <t>22:21</t>
         </is>
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D473" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E473" t="inlineStr">
         <is>
@@ -12173,21 +12173,21 @@
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>22:11:55</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>22:32</t>
+          <t>22:22</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D474" t="n">
-        <v>109</v>
+        <v>11</v>
       </c>
       <c r="E474" t="inlineStr">
         <is>
@@ -12203,16 +12203,16 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>22:38</t>
+          <t>22:24</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D475" t="n">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="E475" t="inlineStr">
         <is>
@@ -12223,21 +12223,21 @@
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>22:11:55</t>
         </is>
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>22:39</t>
+          <t>22:31</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D476" t="n">
-        <v>116</v>
+        <v>20</v>
       </c>
       <c r="E476" t="inlineStr">
         <is>
@@ -12248,23 +12248,298 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>20:59:36</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
         <is>
+          <t>22:32</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D477" t="n">
+        <v>109</v>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>22:38</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D478" t="n">
+        <v>27</v>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>20:43:05</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>22:39</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D479" t="n">
+        <v>116</v>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>22:50</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D480" t="n">
+        <v>39</v>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>22:53</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D481" t="n">
+        <v>42</v>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
           <t>22:57</t>
         </is>
       </c>
-      <c r="C477" t="inlineStr">
+      <c r="C482" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D477" t="n">
-        <v>118</v>
-      </c>
-      <c r="E477" t="inlineStr">
+      <c r="D482" t="n">
+        <v>46</v>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>23:07</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D483" t="n">
+        <v>56</v>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>23:17</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D484" t="n">
+        <v>66</v>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>23:22</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D485" t="n">
+        <v>71</v>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>23:25</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D486" t="n">
+        <v>74</v>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>23:37</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D487" t="n">
+        <v>86</v>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>23:52</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D488" t="n">
+        <v>101</v>
+      </c>
+      <c r="E488" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -12281,7 +12556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12294,14 +12569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:59:36</t>
+          <t>Última actualización: 22:11:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 59</t>
+          <t>Total filas: 60</t>
         </is>
       </c>
     </row>
@@ -12670,7 +12945,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -12695,7 +12970,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -13785,7 +14060,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>20:59:36</t>
+          <t>22:11:55</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -13799,9 +14074,34 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>118</v>
+        <v>46</v>
       </c>
       <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>23:37</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>86</v>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -13831,7 +14131,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:59:36</t>
+          <t>Última actualización: 22:11:55</t>
         </is>
       </c>
     </row>
@@ -15322,7 +15622,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>20:59:36</t>
+          <t>22:11:55</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -15336,7 +15636,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -15347,7 +15647,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>20:59:36</t>
+          <t>22:11:55</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -15361,7 +15661,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>82</v>
+        <v>10</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4236
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-14.xlsx
+++ b/data/horarios-141-2026-08-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E488"/>
+  <dimension ref="A1:E492"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 22:11:55</t>
+          <t>Última actualización: 23:19:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 483</t>
+          <t>Total filas: 487</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:50:36</t>
+          <t>05:55:52</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>05:55:52</t>
+          <t>06:50:36</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>07:45:53</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>07:45:53</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>09:07:23</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:07:23</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:33:25</t>
+          <t>10:34:33</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>10:34:33</t>
+          <t>11:33:25</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>12:24:23</t>
+          <t>13:10:41</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>13:10:41</t>
+          <t>12:24:23</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D297" t="n">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>16:52:07</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7983,11 +7983,11 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8023,7 +8023,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>16:52:07</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -8033,11 +8033,11 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8123,7 +8123,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>16:07:47</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -8133,11 +8133,11 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,7 +8148,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>16:07:47</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -8158,11 +8158,11 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D336" t="n">
@@ -8773,7 +8773,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -8783,11 +8783,11 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,7 +8798,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -8808,11 +8808,11 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8948,7 +8948,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>17:48:37</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -8958,11 +8958,11 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>17:48:37</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -9008,11 +9008,11 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>17:19:27</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,7 +9098,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>17:19:27</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -9108,11 +9108,11 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9783,7 +9783,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D378" t="n">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D379" t="n">
@@ -9848,7 +9848,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>18:34:49</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
@@ -9858,11 +9858,11 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9873,7 +9873,7 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>18:34:49</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
@@ -9883,11 +9883,11 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E382" t="inlineStr">
         <is>
@@ -10123,7 +10123,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:06:31</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -10133,11 +10133,11 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,7 +10148,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>18:06:31</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -10158,11 +10158,11 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>72</v>
+        <v>8</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10498,7 +10498,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -10508,11 +10508,11 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="E407" t="inlineStr">
         <is>
@@ -10523,7 +10523,7 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
@@ -10533,11 +10533,11 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="E408" t="inlineStr">
         <is>
@@ -10748,7 +10748,7 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>19:40:57</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
@@ -10758,11 +10758,11 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D417" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="E417" t="inlineStr">
         <is>
@@ -10773,7 +10773,7 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>19:40:57</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
@@ -10783,11 +10783,11 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D418" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="E418" t="inlineStr">
         <is>
@@ -10798,7 +10798,7 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:59:51</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
@@ -10808,11 +10808,11 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>73</v>
+        <v>7</v>
       </c>
       <c r="E419" t="inlineStr">
         <is>
@@ -10823,7 +10823,7 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>19:59:51</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
@@ -10833,11 +10833,11 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D420" t="n">
-        <v>7</v>
+        <v>73</v>
       </c>
       <c r="E420" t="inlineStr">
         <is>
@@ -10998,7 +10998,7 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>19:10:39</t>
+          <t>18:53:06</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
@@ -11008,11 +11008,11 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D427" t="n">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="E427" t="inlineStr">
         <is>
@@ -11023,7 +11023,7 @@
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>18:53:06</t>
+          <t>19:10:39</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
@@ -11033,11 +11033,11 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D428" t="n">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="E428" t="inlineStr">
         <is>
@@ -11673,7 +11673,7 @@
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>20:43:05</t>
+          <t>20:59:36</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
@@ -11683,11 +11683,11 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D454" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E454" t="inlineStr">
         <is>
@@ -11698,7 +11698,7 @@
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>20:59:36</t>
+          <t>20:43:05</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
@@ -11708,11 +11708,11 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D455" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E455" t="inlineStr">
         <is>
@@ -12473,21 +12473,21 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>22:11:55</t>
+          <t>23:19:04</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>23:25</t>
+          <t>23:23</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D486" t="n">
-        <v>74</v>
+        <v>4</v>
       </c>
       <c r="E486" t="inlineStr">
         <is>
@@ -12503,16 +12503,16 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>23:37</t>
+          <t>23:25</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D487" t="n">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="E487" t="inlineStr">
         <is>
@@ -12523,23 +12523,123 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
+          <t>23:19:04</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>23:26</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D488" t="n">
+        <v>7</v>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
           <t>22:11:55</t>
         </is>
       </c>
-      <c r="B488" t="inlineStr">
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>23:37</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D489" t="n">
+        <v>86</v>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>23:19:04</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>23:38</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D490" t="n">
+        <v>19</v>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>22:11:55</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
         <is>
           <t>23:52</t>
         </is>
       </c>
-      <c r="C488" t="inlineStr">
+      <c r="C491" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D488" t="n">
+      <c r="D491" t="n">
         <v>101</v>
       </c>
-      <c r="E488" t="inlineStr">
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>23:19:04</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>23:53</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D492" t="n">
+        <v>34</v>
+      </c>
+      <c r="E492" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -12556,7 +12656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12569,14 +12669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 22:11:55</t>
+          <t>Última actualización: 23:19:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 60</t>
+          <t>Total filas: 61</t>
         </is>
       </c>
     </row>
@@ -12945,7 +13045,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -12970,7 +13070,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -14102,6 +14202,31 @@
         <v>86</v>
       </c>
       <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>23:19:04</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>23:38</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>19</v>
+      </c>
+      <c r="E66" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -14131,7 +14256,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 22:11:55</t>
+          <t>Última actualización: 23:19:04</t>
         </is>
       </c>
     </row>

</xml_diff>